<commit_message>
ajustes dashboard crm tipo operacion y matriz mensual
</commit_message>
<xml_diff>
--- a/BD CRM 14042026.xlsx
+++ b/BD CRM 14042026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tractocar-my.sharepoint.com/personal/avera_tractocar_com/Documents/Team Comercial/CRM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarias\Desktop\CRM\crm_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1772" documentId="8_{F2A5B7CE-E8D2-40BD-8C9A-6BB22E881C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AD9E9BC-55F6-4A1A-AAF8-C4686E62765B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15EF789-C2BE-4E21-823E-10F37E241A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E68C7C40-B1B6-4540-8438-F3ACB83D4A52}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="333" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -32,8 +32,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -2036,12 +2034,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;\ #,##0"/>
-    <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2213,7 +2210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -2279,12 +2276,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2294,31 +2285,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2917,7 +2890,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
+      <numFmt numFmtId="19" formatCode="d/mm/yyyy"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -2957,7 +2930,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
+      <numFmt numFmtId="19" formatCode="d/mm/yyyy"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -3029,7 +3002,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
+      <numFmt numFmtId="19" formatCode="d/mm/yyyy"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -3101,7 +3074,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
+      <numFmt numFmtId="19" formatCode="d/mm/yyyy"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -3165,13 +3138,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14999847407452621"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color theme="0" tint="-0.14999847407452621"/>
@@ -3207,6 +3173,13 @@
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -11176,7 +11149,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{85491199-660D-426C-9385-E7AF8A153D4E}" name="TablaDinámica1" cacheId="333" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{85491199-660D-426C-9385-E7AF8A153D4E}" name="TablaDinámica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:D76" firstHeaderRow="1" firstDataRow="1" firstDataCol="4" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="23">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -11702,11 +11675,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3B0873A0-70FC-403E-BC89-61BBA66734E5}" name="Tabla1" displayName="Tabla1" ref="A1:X342" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28" headerRowBorderDxfId="26" tableBorderDxfId="27" totalsRowBorderDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3B0873A0-70FC-403E-BC89-61BBA66734E5}" name="Tabla1" displayName="Tabla1" ref="A1:X342" totalsRowShown="0" headerRowDxfId="29" dataDxfId="27" headerRowBorderDxfId="28" tableBorderDxfId="26" totalsRowBorderDxfId="25">
   <autoFilter ref="A1:X342" xr:uid="{3B0873A0-70FC-403E-BC89-61BBA66734E5}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:X336">
-    <sortCondition ref="B1:B336"/>
-  </sortState>
   <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{1F3C2F4B-3283-49FD-BF01-C0A6044E1803}" name="Canal" dataDxfId="24"/>
     <tableColumn id="2" xr3:uid="{2494748F-B628-40E5-ABB1-1EB355F949F8}" name="Fecha Ingreso Solicitud" dataDxfId="23"/>
@@ -11820,7 +11790,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -12117,7 +12087,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C5770D-06F6-4265-B815-90352D3707BC}">
   <dimension ref="A1:X342"/>
-  <sheetFormatPr defaultColWidth="17.42578125" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="17.42578125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="12" width="17.42578125" style="12"/>
     <col min="13" max="13" width="21.42578125" style="12" customWidth="1"/>
@@ -12127,7 +12097,7 @@
     <col min="22" max="16384" width="17.42578125" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="6" customFormat="1" ht="46.5">
+    <row r="1" spans="1:24" s="6" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -12201,7 +12171,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>24</v>
       </c>
@@ -12212,7 +12182,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="D2" s="8">
-        <v>45692</v>
+        <v>46057</v>
       </c>
       <c r="E2" s="9">
         <v>0.33333333333333331</v>
@@ -12261,7 +12231,7 @@
       <c r="U2" s="11"/>
       <c r="V2" s="11"/>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>24</v>
       </c>
@@ -12272,7 +12242,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="D3" s="8">
-        <v>45694</v>
+        <v>46059</v>
       </c>
       <c r="E3" s="9">
         <v>0.33333333333333331</v>
@@ -12317,7 +12287,7 @@
       <c r="U3" s="11"/>
       <c r="V3" s="11"/>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>37</v>
       </c>
@@ -12375,7 +12345,7 @@
       <c r="U4" s="11"/>
       <c r="V4" s="11"/>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>24</v>
       </c>
@@ -12386,7 +12356,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="D5" s="8">
-        <v>45700</v>
+        <v>46065</v>
       </c>
       <c r="E5" s="9">
         <v>0.33333333333333331</v>
@@ -12431,7 +12401,7 @@
       <c r="U5" s="11"/>
       <c r="V5" s="11"/>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>24</v>
       </c>
@@ -12487,7 +12457,7 @@
       <c r="U6" s="11"/>
       <c r="V6" s="11"/>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>37</v>
       </c>
@@ -12543,7 +12513,7 @@
       <c r="U7" s="11"/>
       <c r="V7" s="11"/>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>24</v>
       </c>
@@ -12603,7 +12573,7 @@
       <c r="U8" s="11"/>
       <c r="V8" s="11"/>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>24</v>
       </c>
@@ -12659,7 +12629,7 @@
       <c r="U9" s="11"/>
       <c r="V9" s="11"/>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>37</v>
       </c>
@@ -12719,7 +12689,7 @@
       <c r="U10" s="11"/>
       <c r="V10" s="11"/>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>24</v>
       </c>
@@ -12767,7 +12737,7 @@
       <c r="U11" s="11"/>
       <c r="V11" s="11"/>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>24</v>
       </c>
@@ -12815,7 +12785,7 @@
       <c r="U12" s="14"/>
       <c r="V12" s="11"/>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>24</v>
       </c>
@@ -12871,7 +12841,7 @@
       <c r="U13" s="11"/>
       <c r="V13" s="11"/>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>24</v>
       </c>
@@ -12919,7 +12889,7 @@
       <c r="U14" s="11"/>
       <c r="V14" s="11"/>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>24</v>
       </c>
@@ -12967,7 +12937,7 @@
       <c r="U15" s="14"/>
       <c r="V15" s="11"/>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>24</v>
       </c>
@@ -13027,7 +12997,7 @@
       <c r="U16" s="11"/>
       <c r="V16" s="11"/>
     </row>
-    <row r="17" spans="1:22">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>24</v>
       </c>
@@ -13077,7 +13047,7 @@
       <c r="U17" s="11"/>
       <c r="V17" s="11"/>
     </row>
-    <row r="18" spans="1:22">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>24</v>
       </c>
@@ -13135,7 +13105,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:22">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>24</v>
       </c>
@@ -13179,7 +13149,7 @@
       <c r="U19" s="11"/>
       <c r="V19" s="11"/>
     </row>
-    <row r="20" spans="1:22">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>78</v>
       </c>
@@ -13227,7 +13197,7 @@
       <c r="U20" s="11"/>
       <c r="V20" s="11"/>
     </row>
-    <row r="21" spans="1:22">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>24</v>
       </c>
@@ -13281,7 +13251,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:22">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>24</v>
       </c>
@@ -13335,7 +13305,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:22">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>24</v>
       </c>
@@ -13385,7 +13355,7 @@
       <c r="U23" s="11"/>
       <c r="V23" s="11"/>
     </row>
-    <row r="24" spans="1:22">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>24</v>
       </c>
@@ -13443,7 +13413,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="25" spans="1:22">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>24</v>
       </c>
@@ -13493,7 +13463,7 @@
       <c r="U25" s="11"/>
       <c r="V25" s="11"/>
     </row>
-    <row r="26" spans="1:22">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>24</v>
       </c>
@@ -13541,7 +13511,7 @@
       <c r="U26" s="11"/>
       <c r="V26" s="11"/>
     </row>
-    <row r="27" spans="1:22">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>24</v>
       </c>
@@ -13589,7 +13559,7 @@
       <c r="U27" s="11"/>
       <c r="V27" s="11"/>
     </row>
-    <row r="28" spans="1:22">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>24</v>
       </c>
@@ -13643,7 +13613,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:22">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>24</v>
       </c>
@@ -13697,7 +13667,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="30" spans="1:22">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>24</v>
       </c>
@@ -13745,7 +13715,7 @@
       <c r="U30" s="11"/>
       <c r="V30" s="11"/>
     </row>
-    <row r="31" spans="1:22">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>24</v>
       </c>
@@ -13771,7 +13741,7 @@
       </c>
       <c r="J31" s="10"/>
       <c r="K31" s="10"/>
-      <c r="L31" s="29" t="s">
+      <c r="L31" s="27" t="s">
         <v>80</v>
       </c>
       <c r="M31" s="10" t="s">
@@ -13793,7 +13763,7 @@
       <c r="U31" s="11"/>
       <c r="V31" s="11"/>
     </row>
-    <row r="32" spans="1:22">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>24</v>
       </c>
@@ -13855,7 +13825,7 @@
       <c r="U32" s="11"/>
       <c r="V32" s="11"/>
     </row>
-    <row r="33" spans="1:22">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>24</v>
       </c>
@@ -13899,7 +13869,7 @@
       <c r="U33" s="11"/>
       <c r="V33" s="11"/>
     </row>
-    <row r="34" spans="1:22">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>24</v>
       </c>
@@ -13949,7 +13919,7 @@
       <c r="U34" s="11"/>
       <c r="V34" s="11"/>
     </row>
-    <row r="35" spans="1:22">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>24</v>
       </c>
@@ -14005,7 +13975,7 @@
       <c r="U35" s="11"/>
       <c r="V35" s="11"/>
     </row>
-    <row r="36" spans="1:22">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>24</v>
       </c>
@@ -14063,7 +14033,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="37" spans="1:22">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
         <v>24</v>
       </c>
@@ -14128,7 +14098,7 @@
       </c>
       <c r="V37" s="11"/>
     </row>
-    <row r="38" spans="1:22">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
         <v>24</v>
       </c>
@@ -14176,7 +14146,7 @@
       <c r="U38" s="14"/>
       <c r="V38" s="11"/>
     </row>
-    <row r="39" spans="1:22">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>24</v>
       </c>
@@ -14226,7 +14196,7 @@
       <c r="U39" s="11"/>
       <c r="V39" s="11"/>
     </row>
-    <row r="40" spans="1:22">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>24</v>
       </c>
@@ -14276,7 +14246,7 @@
       <c r="U40" s="11"/>
       <c r="V40" s="11"/>
     </row>
-    <row r="41" spans="1:22">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>24</v>
       </c>
@@ -14326,7 +14296,7 @@
       <c r="U41" s="11"/>
       <c r="V41" s="11"/>
     </row>
-    <row r="42" spans="1:22">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
         <v>24</v>
       </c>
@@ -14376,7 +14346,7 @@
       <c r="U42" s="11"/>
       <c r="V42" s="11"/>
     </row>
-    <row r="43" spans="1:22">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>24</v>
       </c>
@@ -14428,7 +14398,7 @@
       <c r="U43" s="11"/>
       <c r="V43" s="11"/>
     </row>
-    <row r="44" spans="1:22">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>24</v>
       </c>
@@ -14482,7 +14452,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="45" spans="1:22">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>24</v>
       </c>
@@ -14536,7 +14506,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:22">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
         <v>24</v>
       </c>
@@ -14590,7 +14560,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="47" spans="1:22">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>24</v>
       </c>
@@ -14644,7 +14614,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="48" spans="1:22">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>24</v>
       </c>
@@ -14692,7 +14662,7 @@
       <c r="U48" s="11"/>
       <c r="V48" s="11"/>
     </row>
-    <row r="49" spans="1:22">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>24</v>
       </c>
@@ -14740,7 +14710,7 @@
       <c r="U49" s="11"/>
       <c r="V49" s="11"/>
     </row>
-    <row r="50" spans="1:22">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>24</v>
       </c>
@@ -14788,7 +14758,7 @@
       <c r="U50" s="11"/>
       <c r="V50" s="11"/>
     </row>
-    <row r="51" spans="1:22">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>24</v>
       </c>
@@ -14836,7 +14806,7 @@
       <c r="U51" s="11"/>
       <c r="V51" s="11"/>
     </row>
-    <row r="52" spans="1:22">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
         <v>24</v>
       </c>
@@ -14884,7 +14854,7 @@
       <c r="U52" s="11"/>
       <c r="V52" s="11"/>
     </row>
-    <row r="53" spans="1:22">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>24</v>
       </c>
@@ -14932,7 +14902,7 @@
       <c r="U53" s="11"/>
       <c r="V53" s="11"/>
     </row>
-    <row r="54" spans="1:22">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
         <v>24</v>
       </c>
@@ -14980,7 +14950,7 @@
       <c r="U54" s="11"/>
       <c r="V54" s="11"/>
     </row>
-    <row r="55" spans="1:22">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>24</v>
       </c>
@@ -15030,7 +15000,7 @@
       <c r="U55" s="11"/>
       <c r="V55" s="11"/>
     </row>
-    <row r="56" spans="1:22">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
         <v>24</v>
       </c>
@@ -15080,7 +15050,7 @@
       <c r="U56" s="11"/>
       <c r="V56" s="11"/>
     </row>
-    <row r="57" spans="1:22">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>37</v>
       </c>
@@ -15136,7 +15106,7 @@
       <c r="U57" s="11"/>
       <c r="V57" s="11"/>
     </row>
-    <row r="58" spans="1:22">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
         <v>24</v>
       </c>
@@ -15190,7 +15160,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="59" spans="1:22">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>24</v>
       </c>
@@ -15238,7 +15208,7 @@
       <c r="U59" s="14"/>
       <c r="V59" s="11"/>
     </row>
-    <row r="60" spans="1:22">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
         <v>24</v>
       </c>
@@ -15288,7 +15258,7 @@
       <c r="U60" s="11"/>
       <c r="V60" s="11"/>
     </row>
-    <row r="61" spans="1:22">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
         <v>24</v>
       </c>
@@ -15338,7 +15308,7 @@
       <c r="U61" s="11"/>
       <c r="V61" s="11"/>
     </row>
-    <row r="62" spans="1:22">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>24</v>
       </c>
@@ -15386,7 +15356,7 @@
       <c r="U62" s="11"/>
       <c r="V62" s="11"/>
     </row>
-    <row r="63" spans="1:22">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>24</v>
       </c>
@@ -15434,7 +15404,7 @@
       <c r="U63" s="11"/>
       <c r="V63" s="11"/>
     </row>
-    <row r="64" spans="1:22">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>24</v>
       </c>
@@ -15482,7 +15452,7 @@
       <c r="U64" s="14"/>
       <c r="V64" s="11"/>
     </row>
-    <row r="65" spans="1:22">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>24</v>
       </c>
@@ -15534,7 +15504,7 @@
       <c r="U65" s="11"/>
       <c r="V65" s="11"/>
     </row>
-    <row r="66" spans="1:22">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>24</v>
       </c>
@@ -15588,7 +15558,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="67" spans="1:22">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>24</v>
       </c>
@@ -15638,7 +15608,7 @@
       <c r="U67" s="11"/>
       <c r="V67" s="11"/>
     </row>
-    <row r="68" spans="1:22">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>24</v>
       </c>
@@ -15688,7 +15658,7 @@
       <c r="U68" s="11"/>
       <c r="V68" s="11"/>
     </row>
-    <row r="69" spans="1:22">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>24</v>
       </c>
@@ -15738,7 +15708,7 @@
       <c r="U69" s="11"/>
       <c r="V69" s="11"/>
     </row>
-    <row r="70" spans="1:22">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>24</v>
       </c>
@@ -15790,7 +15760,7 @@
       <c r="U70" s="11"/>
       <c r="V70" s="11"/>
     </row>
-    <row r="71" spans="1:22">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>24</v>
       </c>
@@ -15844,7 +15814,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="72" spans="1:22">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>24</v>
       </c>
@@ -15902,7 +15872,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="73" spans="1:22">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>24</v>
       </c>
@@ -15960,7 +15930,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="74" spans="1:22">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
         <v>24</v>
       </c>
@@ -16020,7 +15990,7 @@
       </c>
       <c r="V74" s="11"/>
     </row>
-    <row r="75" spans="1:22">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
         <v>24</v>
       </c>
@@ -16064,7 +16034,7 @@
       <c r="U75" s="11"/>
       <c r="V75" s="11"/>
     </row>
-    <row r="76" spans="1:22">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
         <v>24</v>
       </c>
@@ -16112,7 +16082,7 @@
       <c r="U76" s="14"/>
       <c r="V76" s="11"/>
     </row>
-    <row r="77" spans="1:22">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
         <v>24</v>
       </c>
@@ -16162,7 +16132,7 @@
       <c r="U77" s="11"/>
       <c r="V77" s="11"/>
     </row>
-    <row r="78" spans="1:22">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
         <v>24</v>
       </c>
@@ -16206,7 +16176,7 @@
       <c r="U78" s="11"/>
       <c r="V78" s="11"/>
     </row>
-    <row r="79" spans="1:22">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
         <v>24</v>
       </c>
@@ -16256,7 +16226,7 @@
       <c r="U79" s="11"/>
       <c r="V79" s="11"/>
     </row>
-    <row r="80" spans="1:22">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
         <v>24</v>
       </c>
@@ -16312,7 +16282,7 @@
       <c r="U80" s="11"/>
       <c r="V80" s="11"/>
     </row>
-    <row r="81" spans="1:22">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
         <v>24</v>
       </c>
@@ -16356,7 +16326,7 @@
       <c r="U81" s="11"/>
       <c r="V81" s="11"/>
     </row>
-    <row r="82" spans="1:22">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A82" s="7" t="s">
         <v>24</v>
       </c>
@@ -16404,7 +16374,7 @@
       <c r="U82" s="14"/>
       <c r="V82" s="11"/>
     </row>
-    <row r="83" spans="1:22">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
         <v>24</v>
       </c>
@@ -16458,7 +16428,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="84" spans="1:22">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
         <v>24</v>
       </c>
@@ -16518,7 +16488,7 @@
       <c r="U84" s="11"/>
       <c r="V84" s="11"/>
     </row>
-    <row r="85" spans="1:22">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
         <v>24</v>
       </c>
@@ -16576,7 +16546,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="86" spans="1:22">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A86" s="7" t="s">
         <v>24</v>
       </c>
@@ -16636,7 +16606,7 @@
       </c>
       <c r="V86" s="11"/>
     </row>
-    <row r="87" spans="1:22">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
         <v>24</v>
       </c>
@@ -16686,7 +16656,7 @@
       <c r="U87" s="11"/>
       <c r="V87" s="11"/>
     </row>
-    <row r="88" spans="1:22">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A88" s="7" t="s">
         <v>24</v>
       </c>
@@ -16736,7 +16706,7 @@
       <c r="U88" s="11"/>
       <c r="V88" s="11"/>
     </row>
-    <row r="89" spans="1:22">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
         <v>24</v>
       </c>
@@ -16792,7 +16762,7 @@
       <c r="U89" s="11"/>
       <c r="V89" s="11"/>
     </row>
-    <row r="90" spans="1:22">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A90" s="7" t="s">
         <v>24</v>
       </c>
@@ -16852,7 +16822,7 @@
       </c>
       <c r="V90" s="11"/>
     </row>
-    <row r="91" spans="1:22">
+    <row r="91" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
         <v>24</v>
       </c>
@@ -16902,7 +16872,7 @@
       <c r="U91" s="11"/>
       <c r="V91" s="11"/>
     </row>
-    <row r="92" spans="1:22">
+    <row r="92" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A92" s="7" t="s">
         <v>24</v>
       </c>
@@ -16952,7 +16922,7 @@
       <c r="U92" s="11"/>
       <c r="V92" s="11"/>
     </row>
-    <row r="93" spans="1:22">
+    <row r="93" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
         <v>24</v>
       </c>
@@ -17008,7 +16978,7 @@
       <c r="U93" s="14"/>
       <c r="V93" s="11"/>
     </row>
-    <row r="94" spans="1:22">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A94" s="7" t="s">
         <v>24</v>
       </c>
@@ -17068,7 +17038,7 @@
       <c r="U94" s="11"/>
       <c r="V94" s="11"/>
     </row>
-    <row r="95" spans="1:22">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
         <v>24</v>
       </c>
@@ -17120,7 +17090,7 @@
       <c r="U95" s="11"/>
       <c r="V95" s="11"/>
     </row>
-    <row r="96" spans="1:22">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
         <v>24</v>
       </c>
@@ -17174,7 +17144,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="97" spans="1:24">
+    <row r="97" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
         <v>24</v>
       </c>
@@ -17228,7 +17198,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="98" spans="1:24">
+    <row r="98" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A98" s="7" t="s">
         <v>24</v>
       </c>
@@ -17278,7 +17248,7 @@
       <c r="U98" s="11"/>
       <c r="V98" s="11"/>
     </row>
-    <row r="99" spans="1:24">
+    <row r="99" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
         <v>24</v>
       </c>
@@ -17328,7 +17298,7 @@
       <c r="U99" s="11"/>
       <c r="V99" s="11"/>
     </row>
-    <row r="100" spans="1:24">
+    <row r="100" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
         <v>24</v>
       </c>
@@ -17378,7 +17348,7 @@
       <c r="U100" s="11"/>
       <c r="V100" s="11"/>
     </row>
-    <row r="101" spans="1:24">
+    <row r="101" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
         <v>24</v>
       </c>
@@ -17430,7 +17400,7 @@
       <c r="U101" s="11"/>
       <c r="V101" s="11"/>
     </row>
-    <row r="102" spans="1:24">
+    <row r="102" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
         <v>24</v>
       </c>
@@ -17480,7 +17450,7 @@
       <c r="U102" s="11"/>
       <c r="V102" s="11"/>
     </row>
-    <row r="103" spans="1:24">
+    <row r="103" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
         <v>24</v>
       </c>
@@ -17536,7 +17506,7 @@
       <c r="U103" s="11"/>
       <c r="V103" s="11"/>
     </row>
-    <row r="104" spans="1:24">
+    <row r="104" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A104" s="7" t="s">
         <v>24</v>
       </c>
@@ -17594,7 +17564,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="105" spans="1:24">
+    <row r="105" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
         <v>24</v>
       </c>
@@ -17652,7 +17622,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="106" spans="1:24">
+    <row r="106" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
         <v>24</v>
       </c>
@@ -17708,7 +17678,7 @@
       <c r="U106" s="11"/>
       <c r="V106" s="11"/>
     </row>
-    <row r="107" spans="1:24">
+    <row r="107" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
         <v>37</v>
       </c>
@@ -17719,7 +17689,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="D107" s="8">
-        <v>45739</v>
+        <v>46104</v>
       </c>
       <c r="E107" s="9">
         <v>0.33333333333333331</v>
@@ -17778,7 +17748,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="108" spans="1:24">
+    <row r="108" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A108" s="7" t="s">
         <v>24</v>
       </c>
@@ -17828,7 +17798,7 @@
       <c r="U108" s="11"/>
       <c r="V108" s="11"/>
     </row>
-    <row r="109" spans="1:24">
+    <row r="109" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
         <v>24</v>
       </c>
@@ -17878,7 +17848,7 @@
       <c r="U109" s="11"/>
       <c r="V109" s="11"/>
     </row>
-    <row r="110" spans="1:24">
+    <row r="110" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A110" s="7" t="s">
         <v>24</v>
       </c>
@@ -17926,7 +17896,7 @@
       <c r="U110" s="11"/>
       <c r="V110" s="11"/>
     </row>
-    <row r="111" spans="1:24">
+    <row r="111" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
         <v>24</v>
       </c>
@@ -17978,7 +17948,7 @@
       <c r="U111" s="11"/>
       <c r="V111" s="11"/>
     </row>
-    <row r="112" spans="1:24">
+    <row r="112" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A112" s="7" t="s">
         <v>24</v>
       </c>
@@ -18032,7 +18002,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="113" spans="1:22">
+    <row r="113" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
         <v>24</v>
       </c>
@@ -18082,7 +18052,7 @@
       <c r="U113" s="11"/>
       <c r="V113" s="11"/>
     </row>
-    <row r="114" spans="1:22">
+    <row r="114" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A114" s="7" t="s">
         <v>24</v>
       </c>
@@ -18130,7 +18100,7 @@
       <c r="U114" s="11"/>
       <c r="V114" s="11"/>
     </row>
-    <row r="115" spans="1:22">
+    <row r="115" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
         <v>194</v>
       </c>
@@ -18178,7 +18148,7 @@
       <c r="U115" s="11"/>
       <c r="V115" s="11"/>
     </row>
-    <row r="116" spans="1:22">
+    <row r="116" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A116" s="7" t="s">
         <v>24</v>
       </c>
@@ -18228,7 +18198,7 @@
       <c r="U116" s="11"/>
       <c r="V116" s="11"/>
     </row>
-    <row r="117" spans="1:22">
+    <row r="117" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
         <v>24</v>
       </c>
@@ -18274,7 +18244,7 @@
       <c r="U117" s="11"/>
       <c r="V117" s="11"/>
     </row>
-    <row r="118" spans="1:22">
+    <row r="118" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A118" s="7" t="s">
         <v>37</v>
       </c>
@@ -18334,7 +18304,7 @@
       <c r="U118" s="11"/>
       <c r="V118" s="11"/>
     </row>
-    <row r="119" spans="1:22">
+    <row r="119" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
         <v>37</v>
       </c>
@@ -18394,7 +18364,7 @@
       <c r="U119" s="11"/>
       <c r="V119" s="11"/>
     </row>
-    <row r="120" spans="1:22">
+    <row r="120" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A120" s="7" t="s">
         <v>24</v>
       </c>
@@ -18448,7 +18418,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="121" spans="1:22">
+    <row r="121" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A121" s="7" t="s">
         <v>24</v>
       </c>
@@ -18502,7 +18472,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="122" spans="1:22">
+    <row r="122" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A122" s="7" t="s">
         <v>24</v>
       </c>
@@ -18558,7 +18528,7 @@
       <c r="U122" s="11"/>
       <c r="V122" s="11"/>
     </row>
-    <row r="123" spans="1:22">
+    <row r="123" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A123" s="7" t="s">
         <v>24</v>
       </c>
@@ -18608,7 +18578,7 @@
       <c r="U123" s="11"/>
       <c r="V123" s="11"/>
     </row>
-    <row r="124" spans="1:22">
+    <row r="124" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A124" s="7" t="s">
         <v>24</v>
       </c>
@@ -18658,7 +18628,7 @@
       <c r="U124" s="11"/>
       <c r="V124" s="11"/>
     </row>
-    <row r="125" spans="1:22">
+    <row r="125" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
         <v>24</v>
       </c>
@@ -18708,7 +18678,7 @@
       <c r="U125" s="11"/>
       <c r="V125" s="11"/>
     </row>
-    <row r="126" spans="1:22">
+    <row r="126" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A126" s="7" t="s">
         <v>24</v>
       </c>
@@ -18760,7 +18730,7 @@
       <c r="U126" s="11"/>
       <c r="V126" s="11"/>
     </row>
-    <row r="127" spans="1:22">
+    <row r="127" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
         <v>24</v>
       </c>
@@ -18804,7 +18774,7 @@
       <c r="U127" s="11"/>
       <c r="V127" s="11"/>
     </row>
-    <row r="128" spans="1:22">
+    <row r="128" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A128" s="7" t="s">
         <v>24</v>
       </c>
@@ -18858,7 +18828,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="129" spans="1:22">
+    <row r="129" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
         <v>24</v>
       </c>
@@ -18908,7 +18878,7 @@
       <c r="U129" s="11"/>
       <c r="V129" s="11"/>
     </row>
-    <row r="130" spans="1:22">
+    <row r="130" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A130" s="7" t="s">
         <v>24</v>
       </c>
@@ -18960,7 +18930,7 @@
       <c r="U130" s="11"/>
       <c r="V130" s="11"/>
     </row>
-    <row r="131" spans="1:22">
+    <row r="131" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
         <v>24</v>
       </c>
@@ -19014,7 +18984,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="132" spans="1:22">
+    <row r="132" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A132" s="7" t="s">
         <v>24</v>
       </c>
@@ -19066,7 +19036,7 @@
       <c r="U132" s="11"/>
       <c r="V132" s="11"/>
     </row>
-    <row r="133" spans="1:22">
+    <row r="133" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A133" s="7" t="s">
         <v>24</v>
       </c>
@@ -19122,7 +19092,7 @@
       <c r="U133" s="11"/>
       <c r="V133" s="11"/>
     </row>
-    <row r="134" spans="1:22">
+    <row r="134" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A134" s="7" t="s">
         <v>24</v>
       </c>
@@ -19178,7 +19148,7 @@
       <c r="U134" s="11"/>
       <c r="V134" s="11"/>
     </row>
-    <row r="135" spans="1:22">
+    <row r="135" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
         <v>24</v>
       </c>
@@ -19228,7 +19198,7 @@
       <c r="U135" s="11"/>
       <c r="V135" s="11"/>
     </row>
-    <row r="136" spans="1:22">
+    <row r="136" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A136" s="7" t="s">
         <v>24</v>
       </c>
@@ -19282,7 +19252,7 @@
       <c r="U136" s="11"/>
       <c r="V136" s="11"/>
     </row>
-    <row r="137" spans="1:22">
+    <row r="137" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
         <v>24</v>
       </c>
@@ -19336,7 +19306,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="138" spans="1:22">
+    <row r="138" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A138" s="7" t="s">
         <v>24</v>
       </c>
@@ -19392,7 +19362,7 @@
       <c r="U138" s="11"/>
       <c r="V138" s="11"/>
     </row>
-    <row r="139" spans="1:22">
+    <row r="139" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
         <v>24</v>
       </c>
@@ -19442,7 +19412,7 @@
       <c r="U139" s="11"/>
       <c r="V139" s="11"/>
     </row>
-    <row r="140" spans="1:22">
+    <row r="140" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A140" s="7" t="s">
         <v>194</v>
       </c>
@@ -19490,7 +19460,7 @@
       <c r="U140" s="11"/>
       <c r="V140" s="11"/>
     </row>
-    <row r="141" spans="1:22">
+    <row r="141" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A141" s="7" t="s">
         <v>24</v>
       </c>
@@ -19546,7 +19516,7 @@
       <c r="U141" s="14"/>
       <c r="V141" s="11"/>
     </row>
-    <row r="142" spans="1:22">
+    <row r="142" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A142" s="7" t="s">
         <v>24</v>
       </c>
@@ -19596,7 +19566,7 @@
       <c r="U142" s="11"/>
       <c r="V142" s="11"/>
     </row>
-    <row r="143" spans="1:22">
+    <row r="143" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
         <v>24</v>
       </c>
@@ -19646,7 +19616,7 @@
       <c r="U143" s="11"/>
       <c r="V143" s="11"/>
     </row>
-    <row r="144" spans="1:22">
+    <row r="144" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A144" s="7" t="s">
         <v>24</v>
       </c>
@@ -19700,7 +19670,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="145" spans="1:22">
+    <row r="145" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A145" s="7" t="s">
         <v>24</v>
       </c>
@@ -19756,7 +19726,7 @@
       <c r="U145" s="14"/>
       <c r="V145" s="11"/>
     </row>
-    <row r="146" spans="1:22">
+    <row r="146" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A146" s="7" t="s">
         <v>24</v>
       </c>
@@ -19810,7 +19780,7 @@
       <c r="U146" s="19"/>
       <c r="V146" s="11"/>
     </row>
-    <row r="147" spans="1:22">
+    <row r="147" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A147" s="7" t="s">
         <v>24</v>
       </c>
@@ -19858,7 +19828,7 @@
       <c r="U147" s="11"/>
       <c r="V147" s="11"/>
     </row>
-    <row r="148" spans="1:22">
+    <row r="148" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A148" s="7" t="s">
         <v>24</v>
       </c>
@@ -19908,7 +19878,7 @@
       <c r="U148" s="11"/>
       <c r="V148" s="11"/>
     </row>
-    <row r="149" spans="1:22">
+    <row r="149" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A149" s="7" t="s">
         <v>24</v>
       </c>
@@ -19958,7 +19928,7 @@
       <c r="U149" s="11"/>
       <c r="V149" s="11"/>
     </row>
-    <row r="150" spans="1:22">
+    <row r="150" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A150" s="7" t="s">
         <v>24</v>
       </c>
@@ -20008,7 +19978,7 @@
       <c r="U150" s="11"/>
       <c r="V150" s="11"/>
     </row>
-    <row r="151" spans="1:22">
+    <row r="151" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A151" s="7" t="s">
         <v>24</v>
       </c>
@@ -20066,7 +20036,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="152" spans="1:22">
+    <row r="152" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A152" s="7" t="s">
         <v>24</v>
       </c>
@@ -20116,7 +20086,7 @@
       <c r="U152" s="11"/>
       <c r="V152" s="11"/>
     </row>
-    <row r="153" spans="1:22">
+    <row r="153" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A153" s="7" t="s">
         <v>24</v>
       </c>
@@ -20176,7 +20146,7 @@
       </c>
       <c r="V153" s="11"/>
     </row>
-    <row r="154" spans="1:22">
+    <row r="154" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A154" s="7" t="s">
         <v>24</v>
       </c>
@@ -20228,7 +20198,7 @@
       <c r="U154" s="11"/>
       <c r="V154" s="11"/>
     </row>
-    <row r="155" spans="1:22">
+    <row r="155" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A155" s="7" t="s">
         <v>24</v>
       </c>
@@ -20278,7 +20248,7 @@
       <c r="U155" s="11"/>
       <c r="V155" s="11"/>
     </row>
-    <row r="156" spans="1:22">
+    <row r="156" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A156" s="7" t="s">
         <v>24</v>
       </c>
@@ -20330,7 +20300,7 @@
       <c r="U156" s="11"/>
       <c r="V156" s="11"/>
     </row>
-    <row r="157" spans="1:22">
+    <row r="157" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A157" s="7" t="s">
         <v>24</v>
       </c>
@@ -20384,7 +20354,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="158" spans="1:22">
+    <row r="158" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A158" s="7" t="s">
         <v>24</v>
       </c>
@@ -20432,7 +20402,7 @@
       <c r="U158" s="11"/>
       <c r="V158" s="11"/>
     </row>
-    <row r="159" spans="1:22">
+    <row r="159" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A159" s="7" t="s">
         <v>24</v>
       </c>
@@ -20482,7 +20452,7 @@
       <c r="U159" s="11"/>
       <c r="V159" s="11"/>
     </row>
-    <row r="160" spans="1:22">
+    <row r="160" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A160" s="7" t="s">
         <v>24</v>
       </c>
@@ -20534,7 +20504,7 @@
       <c r="U160" s="11"/>
       <c r="V160" s="11"/>
     </row>
-    <row r="161" spans="1:22">
+    <row r="161" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A161" s="7" t="s">
         <v>24</v>
       </c>
@@ -20588,7 +20558,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="162" spans="1:22">
+    <row r="162" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A162" s="7" t="s">
         <v>24</v>
       </c>
@@ -20642,7 +20612,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="163" spans="1:22">
+    <row r="163" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A163" s="7" t="s">
         <v>24</v>
       </c>
@@ -20692,7 +20662,7 @@
       <c r="U163" s="11"/>
       <c r="V163" s="11"/>
     </row>
-    <row r="164" spans="1:22">
+    <row r="164" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A164" s="7" t="s">
         <v>24</v>
       </c>
@@ -20742,7 +20712,7 @@
       <c r="U164" s="11"/>
       <c r="V164" s="11"/>
     </row>
-    <row r="165" spans="1:22">
+    <row r="165" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A165" s="7" t="s">
         <v>24</v>
       </c>
@@ -20790,7 +20760,7 @@
       <c r="U165" s="11"/>
       <c r="V165" s="11"/>
     </row>
-    <row r="166" spans="1:22">
+    <row r="166" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A166" s="7" t="s">
         <v>194</v>
       </c>
@@ -20842,7 +20812,7 @@
       <c r="U166" s="11"/>
       <c r="V166" s="11"/>
     </row>
-    <row r="167" spans="1:22">
+    <row r="167" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A167" s="7" t="s">
         <v>24</v>
       </c>
@@ -20892,7 +20862,7 @@
       <c r="U167" s="11"/>
       <c r="V167" s="11"/>
     </row>
-    <row r="168" spans="1:22">
+    <row r="168" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A168" s="7" t="s">
         <v>24</v>
       </c>
@@ -20946,7 +20916,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="169" spans="1:22">
+    <row r="169" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A169" s="7" t="s">
         <v>24</v>
       </c>
@@ -20990,7 +20960,7 @@
       <c r="U169" s="11"/>
       <c r="V169" s="11"/>
     </row>
-    <row r="170" spans="1:22">
+    <row r="170" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A170" s="7" t="s">
         <v>24</v>
       </c>
@@ -21040,7 +21010,7 @@
       <c r="U170" s="11"/>
       <c r="V170" s="11"/>
     </row>
-    <row r="171" spans="1:22">
+    <row r="171" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A171" s="7" t="s">
         <v>24</v>
       </c>
@@ -21090,7 +21060,7 @@
       <c r="U171" s="11"/>
       <c r="V171" s="11"/>
     </row>
-    <row r="172" spans="1:22">
+    <row r="172" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A172" s="7" t="s">
         <v>24</v>
       </c>
@@ -21140,7 +21110,7 @@
       <c r="U172" s="11"/>
       <c r="V172" s="11"/>
     </row>
-    <row r="173" spans="1:22">
+    <row r="173" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A173" s="7" t="s">
         <v>24</v>
       </c>
@@ -21198,7 +21168,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="174" spans="1:22">
+    <row r="174" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A174" s="7" t="s">
         <v>24</v>
       </c>
@@ -21246,7 +21216,7 @@
       <c r="U174" s="11"/>
       <c r="V174" s="11"/>
     </row>
-    <row r="175" spans="1:22">
+    <row r="175" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A175" s="7" t="s">
         <v>24</v>
       </c>
@@ -21294,7 +21264,7 @@
       <c r="U175" s="11"/>
       <c r="V175" s="11"/>
     </row>
-    <row r="176" spans="1:22">
+    <row r="176" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A176" s="7" t="s">
         <v>24</v>
       </c>
@@ -21348,7 +21318,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="177" spans="1:24">
+    <row r="177" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A177" s="7" t="s">
         <v>24</v>
       </c>
@@ -21396,7 +21366,7 @@
       <c r="U177" s="11"/>
       <c r="V177" s="11"/>
     </row>
-    <row r="178" spans="1:24">
+    <row r="178" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A178" s="7" t="s">
         <v>24</v>
       </c>
@@ -21444,7 +21414,7 @@
       <c r="U178" s="11"/>
       <c r="V178" s="11"/>
     </row>
-    <row r="179" spans="1:24">
+    <row r="179" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A179" s="7" t="s">
         <v>24</v>
       </c>
@@ -21494,7 +21464,7 @@
       <c r="U179" s="11"/>
       <c r="V179" s="11"/>
     </row>
-    <row r="180" spans="1:24">
+    <row r="180" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A180" s="7" t="s">
         <v>24</v>
       </c>
@@ -21544,7 +21514,7 @@
       <c r="U180" s="11"/>
       <c r="V180" s="11"/>
     </row>
-    <row r="181" spans="1:24">
+    <row r="181" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A181" s="7" t="s">
         <v>24</v>
       </c>
@@ -21592,7 +21562,7 @@
       <c r="U181" s="11"/>
       <c r="V181" s="11"/>
     </row>
-    <row r="182" spans="1:24">
+    <row r="182" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A182" s="7" t="s">
         <v>24</v>
       </c>
@@ -21642,7 +21612,7 @@
       <c r="U182" s="11"/>
       <c r="V182" s="11"/>
     </row>
-    <row r="183" spans="1:24">
+    <row r="183" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A183" s="7" t="s">
         <v>24</v>
       </c>
@@ -21698,7 +21668,7 @@
       <c r="U183" s="11"/>
       <c r="V183" s="11"/>
     </row>
-    <row r="184" spans="1:24">
+    <row r="184" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A184" s="7" t="s">
         <v>24</v>
       </c>
@@ -21754,7 +21724,7 @@
       <c r="U184" s="11"/>
       <c r="V184" s="11"/>
     </row>
-    <row r="185" spans="1:24">
+    <row r="185" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A185" s="7" t="s">
         <v>24</v>
       </c>
@@ -21800,7 +21770,7 @@
       <c r="U185" s="11"/>
       <c r="V185" s="11"/>
     </row>
-    <row r="186" spans="1:24">
+    <row r="186" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A186" s="7" t="s">
         <v>24</v>
       </c>
@@ -21848,24 +21818,24 @@
       <c r="U186" s="11"/>
       <c r="V186" s="11"/>
     </row>
-    <row r="187" spans="1:24">
+    <row r="187" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A187" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B187" s="26">
+      <c r="B187" s="8">
         <v>46108</v>
       </c>
       <c r="C187" s="9">
         <v>0.65625</v>
       </c>
-      <c r="D187" s="26">
+      <c r="D187" s="8">
         <v>46122</v>
       </c>
       <c r="E187" s="9">
         <v>0.60624999999999996</v>
       </c>
-      <c r="F187" s="26"/>
-      <c r="G187" s="26"/>
+      <c r="F187" s="8"/>
+      <c r="G187" s="8"/>
       <c r="H187" s="10" t="s">
         <v>38</v>
       </c>
@@ -21912,7 +21882,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="188" spans="1:24">
+    <row r="188" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A188" s="7" t="s">
         <v>24</v>
       </c>
@@ -21962,7 +21932,7 @@
       <c r="U188" s="11"/>
       <c r="V188" s="11"/>
     </row>
-    <row r="189" spans="1:24">
+    <row r="189" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A189" s="7" t="s">
         <v>24</v>
       </c>
@@ -22010,7 +21980,7 @@
       <c r="U189" s="11"/>
       <c r="V189" s="11"/>
     </row>
-    <row r="190" spans="1:24">
+    <row r="190" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A190" s="7" t="s">
         <v>24</v>
       </c>
@@ -22066,7 +22036,7 @@
       <c r="U190" s="11"/>
       <c r="V190" s="11"/>
     </row>
-    <row r="191" spans="1:24">
+    <row r="191" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A191" s="7" t="s">
         <v>24</v>
       </c>
@@ -22118,7 +22088,7 @@
       <c r="U191" s="11"/>
       <c r="V191" s="11"/>
     </row>
-    <row r="192" spans="1:24">
+    <row r="192" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A192" s="7" t="s">
         <v>37</v>
       </c>
@@ -22176,7 +22146,7 @@
       </c>
       <c r="V192" s="11"/>
     </row>
-    <row r="193" spans="1:22">
+    <row r="193" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A193" s="7" t="s">
         <v>24</v>
       </c>
@@ -22224,7 +22194,7 @@
       <c r="U193" s="11"/>
       <c r="V193" s="11"/>
     </row>
-    <row r="194" spans="1:22">
+    <row r="194" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A194" s="7" t="s">
         <v>24</v>
       </c>
@@ -22274,7 +22244,7 @@
       <c r="U194" s="11"/>
       <c r="V194" s="11"/>
     </row>
-    <row r="195" spans="1:22">
+    <row r="195" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A195" s="7" t="s">
         <v>24</v>
       </c>
@@ -22328,7 +22298,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="196" spans="1:22">
+    <row r="196" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A196" s="7" t="s">
         <v>24</v>
       </c>
@@ -22384,7 +22354,7 @@
       <c r="U196" s="14"/>
       <c r="V196" s="11"/>
     </row>
-    <row r="197" spans="1:22">
+    <row r="197" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A197" s="7" t="s">
         <v>24</v>
       </c>
@@ -22440,7 +22410,7 @@
       <c r="U197" s="11"/>
       <c r="V197" s="11"/>
     </row>
-    <row r="198" spans="1:22">
+    <row r="198" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A198" s="7" t="s">
         <v>24</v>
       </c>
@@ -22490,7 +22460,7 @@
       <c r="U198" s="11"/>
       <c r="V198" s="11"/>
     </row>
-    <row r="199" spans="1:22">
+    <row r="199" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A199" s="7" t="s">
         <v>24</v>
       </c>
@@ -22540,7 +22510,7 @@
       <c r="U199" s="11"/>
       <c r="V199" s="11"/>
     </row>
-    <row r="200" spans="1:22">
+    <row r="200" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A200" s="7" t="s">
         <v>24</v>
       </c>
@@ -22590,7 +22560,7 @@
       <c r="U200" s="11"/>
       <c r="V200" s="11"/>
     </row>
-    <row r="201" spans="1:22">
+    <row r="201" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A201" s="7" t="s">
         <v>24</v>
       </c>
@@ -22646,7 +22616,7 @@
       <c r="U201" s="11"/>
       <c r="V201" s="11"/>
     </row>
-    <row r="202" spans="1:22">
+    <row r="202" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A202" s="7" t="s">
         <v>24</v>
       </c>
@@ -22704,7 +22674,7 @@
       <c r="U202" s="14"/>
       <c r="V202" s="11"/>
     </row>
-    <row r="203" spans="1:22">
+    <row r="203" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A203" s="7" t="s">
         <v>24</v>
       </c>
@@ -22762,7 +22732,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="204" spans="1:22">
+    <row r="204" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A204" s="7" t="s">
         <v>24</v>
       </c>
@@ -22808,7 +22778,7 @@
       <c r="U204" s="11"/>
       <c r="V204" s="11"/>
     </row>
-    <row r="205" spans="1:22">
+    <row r="205" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A205" s="7" t="s">
         <v>24</v>
       </c>
@@ -22858,7 +22828,7 @@
       <c r="U205" s="11"/>
       <c r="V205" s="11"/>
     </row>
-    <row r="206" spans="1:22">
+    <row r="206" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A206" s="7" t="s">
         <v>24</v>
       </c>
@@ -22914,7 +22884,7 @@
       <c r="U206" s="11"/>
       <c r="V206" s="11"/>
     </row>
-    <row r="207" spans="1:22">
+    <row r="207" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A207" s="7" t="s">
         <v>24</v>
       </c>
@@ -22964,7 +22934,7 @@
       <c r="U207" s="11"/>
       <c r="V207" s="11"/>
     </row>
-    <row r="208" spans="1:22">
+    <row r="208" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A208" s="7" t="s">
         <v>24</v>
       </c>
@@ -23014,7 +22984,7 @@
       <c r="U208" s="11"/>
       <c r="V208" s="11"/>
     </row>
-    <row r="209" spans="1:22">
+    <row r="209" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A209" s="7" t="s">
         <v>24</v>
       </c>
@@ -23068,7 +23038,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="210" spans="1:22">
+    <row r="210" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A210" s="7" t="s">
         <v>24</v>
       </c>
@@ -23122,7 +23092,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="211" spans="1:22">
+    <row r="211" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A211" s="7" t="s">
         <v>24</v>
       </c>
@@ -23184,7 +23154,7 @@
       <c r="U211" s="11"/>
       <c r="V211" s="11"/>
     </row>
-    <row r="212" spans="1:22">
+    <row r="212" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A212" s="7" t="s">
         <v>24</v>
       </c>
@@ -23230,7 +23200,7 @@
       <c r="U212" s="11"/>
       <c r="V212" s="11"/>
     </row>
-    <row r="213" spans="1:22">
+    <row r="213" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A213" s="7" t="s">
         <v>24</v>
       </c>
@@ -23284,7 +23254,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="214" spans="1:22">
+    <row r="214" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A214" s="7" t="s">
         <v>24</v>
       </c>
@@ -23338,7 +23308,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="215" spans="1:22">
+    <row r="215" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A215" s="7" t="s">
         <v>24</v>
       </c>
@@ -23392,7 +23362,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="216" spans="1:22">
+    <row r="216" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A216" s="7" t="s">
         <v>24</v>
       </c>
@@ -23446,7 +23416,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="217" spans="1:22">
+    <row r="217" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A217" s="7" t="s">
         <v>24</v>
       </c>
@@ -23500,7 +23470,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="218" spans="1:22">
+    <row r="218" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A218" s="7" t="s">
         <v>24</v>
       </c>
@@ -23558,7 +23528,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="219" spans="1:22">
+    <row r="219" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A219" s="7" t="s">
         <v>24</v>
       </c>
@@ -23612,7 +23582,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="220" spans="1:22">
+    <row r="220" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A220" s="7" t="s">
         <v>24</v>
       </c>
@@ -23664,7 +23634,7 @@
       <c r="U220" s="11"/>
       <c r="V220" s="11"/>
     </row>
-    <row r="221" spans="1:22">
+    <row r="221" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A221" s="7" t="s">
         <v>24</v>
       </c>
@@ -23718,7 +23688,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="222" spans="1:22">
+    <row r="222" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A222" s="7" t="s">
         <v>24</v>
       </c>
@@ -23772,7 +23742,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="223" spans="1:22">
+    <row r="223" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A223" s="7" t="s">
         <v>24</v>
       </c>
@@ -23820,7 +23790,7 @@
       <c r="U223" s="11"/>
       <c r="V223" s="11"/>
     </row>
-    <row r="224" spans="1:22">
+    <row r="224" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A224" s="7" t="s">
         <v>24</v>
       </c>
@@ -23870,7 +23840,7 @@
       <c r="U224" s="11"/>
       <c r="V224" s="11"/>
     </row>
-    <row r="225" spans="1:22">
+    <row r="225" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A225" s="7" t="s">
         <v>24</v>
       </c>
@@ -23922,7 +23892,7 @@
       <c r="U225" s="11"/>
       <c r="V225" s="11"/>
     </row>
-    <row r="226" spans="1:22">
+    <row r="226" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A226" s="7" t="s">
         <v>194</v>
       </c>
@@ -23970,7 +23940,7 @@
       <c r="U226" s="11"/>
       <c r="V226" s="11"/>
     </row>
-    <row r="227" spans="1:22">
+    <row r="227" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A227" s="7" t="s">
         <v>24</v>
       </c>
@@ -24024,7 +23994,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="228" spans="1:22">
+    <row r="228" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A228" s="7" t="s">
         <v>24</v>
       </c>
@@ -24078,7 +24048,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="229" spans="1:22">
+    <row r="229" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A229" s="7" t="s">
         <v>24</v>
       </c>
@@ -24132,7 +24102,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="230" spans="1:22">
+    <row r="230" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A230" s="7" t="s">
         <v>24</v>
       </c>
@@ -24180,7 +24150,7 @@
       <c r="U230" s="11"/>
       <c r="V230" s="11"/>
     </row>
-    <row r="231" spans="1:22">
+    <row r="231" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A231" s="7" t="s">
         <v>24</v>
       </c>
@@ -24230,7 +24200,7 @@
       <c r="U231" s="11"/>
       <c r="V231" s="11"/>
     </row>
-    <row r="232" spans="1:22">
+    <row r="232" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A232" s="7" t="s">
         <v>24</v>
       </c>
@@ -24280,7 +24250,7 @@
       <c r="U232" s="11"/>
       <c r="V232" s="11"/>
     </row>
-    <row r="233" spans="1:22">
+    <row r="233" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A233" s="7" t="s">
         <v>24</v>
       </c>
@@ -24332,7 +24302,7 @@
       <c r="U233" s="11"/>
       <c r="V233" s="11"/>
     </row>
-    <row r="234" spans="1:22">
+    <row r="234" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A234" s="7" t="s">
         <v>24</v>
       </c>
@@ -24384,7 +24354,7 @@
       <c r="U234" s="11"/>
       <c r="V234" s="11"/>
     </row>
-    <row r="235" spans="1:22">
+    <row r="235" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A235" s="7" t="s">
         <v>24</v>
       </c>
@@ -24434,7 +24404,7 @@
       <c r="U235" s="11"/>
       <c r="V235" s="11"/>
     </row>
-    <row r="236" spans="1:22">
+    <row r="236" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A236" s="7" t="s">
         <v>24</v>
       </c>
@@ -24490,7 +24460,7 @@
       <c r="U236" s="11"/>
       <c r="V236" s="11"/>
     </row>
-    <row r="237" spans="1:22">
+    <row r="237" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A237" s="7" t="s">
         <v>24</v>
       </c>
@@ -24540,7 +24510,7 @@
       <c r="U237" s="11"/>
       <c r="V237" s="11"/>
     </row>
-    <row r="238" spans="1:22">
+    <row r="238" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A238" s="7" t="s">
         <v>24</v>
       </c>
@@ -24594,7 +24564,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="239" spans="1:22">
+    <row r="239" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A239" s="7" t="s">
         <v>24</v>
       </c>
@@ -24648,7 +24618,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="240" spans="1:22">
+    <row r="240" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A240" s="7" t="s">
         <v>78</v>
       </c>
@@ -24696,7 +24666,7 @@
       <c r="U240" s="14"/>
       <c r="V240" s="11"/>
     </row>
-    <row r="241" spans="1:22">
+    <row r="241" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A241" s="7" t="s">
         <v>24</v>
       </c>
@@ -24752,7 +24722,7 @@
       <c r="U241" s="11"/>
       <c r="V241" s="11"/>
     </row>
-    <row r="242" spans="1:22">
+    <row r="242" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A242" s="7" t="s">
         <v>24</v>
       </c>
@@ -24802,7 +24772,7 @@
       <c r="U242" s="11"/>
       <c r="V242" s="11"/>
     </row>
-    <row r="243" spans="1:22">
+    <row r="243" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A243" s="7" t="s">
         <v>24</v>
       </c>
@@ -24848,7 +24818,7 @@
       <c r="U243" s="11"/>
       <c r="V243" s="11"/>
     </row>
-    <row r="244" spans="1:22">
+    <row r="244" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A244" s="7" t="s">
         <v>24</v>
       </c>
@@ -24898,7 +24868,7 @@
       <c r="U244" s="11"/>
       <c r="V244" s="11"/>
     </row>
-    <row r="245" spans="1:22">
+    <row r="245" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A245" s="7" t="s">
         <v>194</v>
       </c>
@@ -24950,7 +24920,7 @@
       <c r="U245" s="11"/>
       <c r="V245" s="11"/>
     </row>
-    <row r="246" spans="1:22">
+    <row r="246" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A246" s="7" t="s">
         <v>24</v>
       </c>
@@ -25000,7 +24970,7 @@
       <c r="U246" s="11"/>
       <c r="V246" s="11"/>
     </row>
-    <row r="247" spans="1:22">
+    <row r="247" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A247" s="7" t="s">
         <v>24</v>
       </c>
@@ -25050,7 +25020,7 @@
       <c r="U247" s="11"/>
       <c r="V247" s="11"/>
     </row>
-    <row r="248" spans="1:22">
+    <row r="248" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A248" s="7" t="s">
         <v>24</v>
       </c>
@@ -25108,7 +25078,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="249" spans="1:22">
+    <row r="249" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A249" s="7" t="s">
         <v>24</v>
       </c>
@@ -25156,7 +25126,7 @@
       <c r="U249" s="14"/>
       <c r="V249" s="11"/>
     </row>
-    <row r="250" spans="1:22">
+    <row r="250" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A250" s="7" t="s">
         <v>24</v>
       </c>
@@ -25204,7 +25174,7 @@
       <c r="U250" s="19"/>
       <c r="V250" s="19"/>
     </row>
-    <row r="251" spans="1:22">
+    <row r="251" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A251" s="7" t="s">
         <v>24</v>
       </c>
@@ -25254,7 +25224,7 @@
       <c r="U251" s="19"/>
       <c r="V251" s="19"/>
     </row>
-    <row r="252" spans="1:22">
+    <row r="252" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A252" s="7" t="s">
         <v>24</v>
       </c>
@@ -25302,7 +25272,7 @@
       <c r="U252" s="19"/>
       <c r="V252" s="19"/>
     </row>
-    <row r="253" spans="1:22">
+    <row r="253" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A253" s="7" t="s">
         <v>24</v>
       </c>
@@ -25350,7 +25320,7 @@
       <c r="U253" s="22"/>
       <c r="V253" s="19"/>
     </row>
-    <row r="254" spans="1:22">
+    <row r="254" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A254" s="7" t="s">
         <v>24</v>
       </c>
@@ -25404,7 +25374,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="255" spans="1:22">
+    <row r="255" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A255" s="7" t="s">
         <v>24</v>
       </c>
@@ -25458,7 +25428,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="256" spans="1:22">
+    <row r="256" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A256" s="7" t="s">
         <v>24</v>
       </c>
@@ -25512,7 +25482,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="257" spans="1:24">
+    <row r="257" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A257" s="7" t="s">
         <v>37</v>
       </c>
@@ -25584,7 +25554,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="258" spans="1:24">
+    <row r="258" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A258" s="7" t="s">
         <v>24</v>
       </c>
@@ -25634,7 +25604,7 @@
       <c r="U258" s="19"/>
       <c r="V258" s="19"/>
     </row>
-    <row r="259" spans="1:24">
+    <row r="259" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A259" s="7" t="s">
         <v>24</v>
       </c>
@@ -25684,7 +25654,7 @@
       <c r="U259" s="19"/>
       <c r="V259" s="19"/>
     </row>
-    <row r="260" spans="1:24">
+    <row r="260" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A260" s="7" t="s">
         <v>24</v>
       </c>
@@ -25744,7 +25714,7 @@
       </c>
       <c r="V260" s="19"/>
     </row>
-    <row r="261" spans="1:24">
+    <row r="261" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A261" s="7" t="s">
         <v>24</v>
       </c>
@@ -25792,7 +25762,7 @@
       <c r="U261" s="19"/>
       <c r="V261" s="19"/>
     </row>
-    <row r="262" spans="1:24">
+    <row r="262" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A262" s="7" t="s">
         <v>24</v>
       </c>
@@ -25858,7 +25828,7 @@
       </c>
       <c r="V262" s="19"/>
     </row>
-    <row r="263" spans="1:24">
+    <row r="263" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A263" s="7" t="s">
         <v>24</v>
       </c>
@@ -25910,7 +25880,7 @@
       <c r="U263" s="22"/>
       <c r="V263" s="19"/>
     </row>
-    <row r="264" spans="1:24">
+    <row r="264" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A264" s="7" t="s">
         <v>24</v>
       </c>
@@ -25962,7 +25932,7 @@
       <c r="U264" s="19"/>
       <c r="V264" s="19"/>
     </row>
-    <row r="265" spans="1:24">
+    <row r="265" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A265" s="15" t="s">
         <v>24</v>
       </c>
@@ -26016,7 +25986,7 @@
       <c r="U265" s="22"/>
       <c r="V265" s="19"/>
     </row>
-    <row r="266" spans="1:24">
+    <row r="266" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A266" s="15" t="s">
         <v>24</v>
       </c>
@@ -26068,7 +26038,7 @@
       <c r="U266" s="19"/>
       <c r="V266" s="19"/>
     </row>
-    <row r="267" spans="1:24">
+    <row r="267" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A267" s="15" t="s">
         <v>24</v>
       </c>
@@ -26122,7 +26092,7 @@
       <c r="U267" s="22"/>
       <c r="V267" s="19"/>
     </row>
-    <row r="268" spans="1:24">
+    <row r="268" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A268" s="15" t="s">
         <v>24</v>
       </c>
@@ -26174,7 +26144,7 @@
       <c r="U268" s="22"/>
       <c r="V268" s="19"/>
     </row>
-    <row r="269" spans="1:24">
+    <row r="269" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A269" s="15" t="s">
         <v>24</v>
       </c>
@@ -26228,7 +26198,7 @@
       <c r="U269" s="22"/>
       <c r="V269" s="19"/>
     </row>
-    <row r="270" spans="1:24">
+    <row r="270" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A270" s="15" t="s">
         <v>24</v>
       </c>
@@ -26278,7 +26248,7 @@
       <c r="U270" s="22"/>
       <c r="V270" s="19"/>
     </row>
-    <row r="271" spans="1:24">
+    <row r="271" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A271" s="15" t="s">
         <v>24</v>
       </c>
@@ -26332,7 +26302,7 @@
       <c r="U271" s="22"/>
       <c r="V271" s="19"/>
     </row>
-    <row r="272" spans="1:24">
+    <row r="272" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A272" s="15" t="s">
         <v>24</v>
       </c>
@@ -26398,7 +26368,7 @@
       </c>
       <c r="V272" s="19"/>
     </row>
-    <row r="273" spans="1:22">
+    <row r="273" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A273" s="15" t="s">
         <v>24</v>
       </c>
@@ -26452,7 +26422,7 @@
       <c r="U273" s="22"/>
       <c r="V273" s="19"/>
     </row>
-    <row r="274" spans="1:22">
+    <row r="274" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A274" s="15" t="s">
         <v>24</v>
       </c>
@@ -26508,7 +26478,7 @@
       <c r="U274" s="22"/>
       <c r="V274" s="19"/>
     </row>
-    <row r="275" spans="1:22">
+    <row r="275" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A275" s="15" t="s">
         <v>24</v>
       </c>
@@ -26560,7 +26530,7 @@
       <c r="U275" s="19"/>
       <c r="V275" s="19"/>
     </row>
-    <row r="276" spans="1:22">
+    <row r="276" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A276" s="15" t="s">
         <v>24</v>
       </c>
@@ -26610,7 +26580,7 @@
       <c r="U276" s="22"/>
       <c r="V276" s="19"/>
     </row>
-    <row r="277" spans="1:22">
+    <row r="277" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A277" s="15" t="s">
         <v>24</v>
       </c>
@@ -26662,7 +26632,7 @@
       <c r="U277" s="22"/>
       <c r="V277" s="19"/>
     </row>
-    <row r="278" spans="1:22">
+    <row r="278" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A278" s="15" t="s">
         <v>24</v>
       </c>
@@ -26714,7 +26684,7 @@
       <c r="U278" s="19"/>
       <c r="V278" s="19"/>
     </row>
-    <row r="279" spans="1:22">
+    <row r="279" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A279" s="15" t="s">
         <v>24</v>
       </c>
@@ -26768,7 +26738,7 @@
       <c r="U279" s="22"/>
       <c r="V279" s="19"/>
     </row>
-    <row r="280" spans="1:22">
+    <row r="280" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A280" s="15" t="s">
         <v>24</v>
       </c>
@@ -26832,7 +26802,7 @@
       </c>
       <c r="V280" s="19"/>
     </row>
-    <row r="281" spans="1:22">
+    <row r="281" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A281" s="15" t="s">
         <v>24</v>
       </c>
@@ -26890,7 +26860,7 @@
       <c r="U281" s="22"/>
       <c r="V281" s="19"/>
     </row>
-    <row r="282" spans="1:22">
+    <row r="282" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A282" s="15" t="s">
         <v>24</v>
       </c>
@@ -26938,7 +26908,7 @@
       <c r="U282" s="19"/>
       <c r="V282" s="19"/>
     </row>
-    <row r="283" spans="1:22">
+    <row r="283" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A283" s="15" t="s">
         <v>24</v>
       </c>
@@ -26988,17 +26958,17 @@
       <c r="U283" s="19"/>
       <c r="V283" s="19"/>
     </row>
-    <row r="284" spans="1:22">
+    <row r="284" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A284" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="B284" s="31">
+      <c r="B284" s="29">
         <v>46127</v>
       </c>
       <c r="C284" s="17">
         <v>0.88472222222222219</v>
       </c>
-      <c r="D284" s="31">
+      <c r="D284" s="29">
         <v>46128</v>
       </c>
       <c r="E284" s="17">
@@ -27042,17 +27012,17 @@
         <v>444</v>
       </c>
     </row>
-    <row r="285" spans="1:22">
+    <row r="285" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A285" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B285" s="31">
+      <c r="B285" s="29">
         <v>46127</v>
       </c>
       <c r="C285" s="17">
         <v>0.45208333333333334</v>
       </c>
-      <c r="D285" s="31">
+      <c r="D285" s="29">
         <v>46128</v>
       </c>
       <c r="E285" s="17">
@@ -27096,17 +27066,17 @@
       <c r="U285" s="19"/>
       <c r="V285" s="19"/>
     </row>
-    <row r="286" spans="1:22">
+    <row r="286" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A286" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B286" s="31">
+      <c r="B286" s="29">
         <v>46127</v>
       </c>
       <c r="C286" s="17">
         <v>0.31388888888888888</v>
       </c>
-      <c r="D286" s="31">
+      <c r="D286" s="29">
         <v>46128</v>
       </c>
       <c r="E286" s="17">
@@ -27152,7 +27122,7 @@
       <c r="U286" s="19"/>
       <c r="V286" s="19"/>
     </row>
-    <row r="287" spans="1:22">
+    <row r="287" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A287" s="15" t="s">
         <v>24</v>
       </c>
@@ -27162,7 +27132,7 @@
       <c r="C287" s="17">
         <v>0.39166666666666666</v>
       </c>
-      <c r="D287" s="31">
+      <c r="D287" s="29">
         <v>46128</v>
       </c>
       <c r="E287" s="17">
@@ -27206,7 +27176,7 @@
       <c r="U287" s="19"/>
       <c r="V287" s="19"/>
     </row>
-    <row r="288" spans="1:22">
+    <row r="288" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A288" s="15" t="s">
         <v>24</v>
       </c>
@@ -27216,7 +27186,7 @@
       <c r="C288" s="17">
         <v>0.50763888888888886</v>
       </c>
-      <c r="D288" s="31">
+      <c r="D288" s="29">
         <v>46128</v>
       </c>
       <c r="E288" s="17">
@@ -27262,7 +27232,7 @@
       <c r="U288" s="19"/>
       <c r="V288" s="19"/>
     </row>
-    <row r="289" spans="1:22">
+    <row r="289" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A289" s="15" t="s">
         <v>24</v>
       </c>
@@ -27314,7 +27284,7 @@
       <c r="U289" s="19"/>
       <c r="V289" s="19"/>
     </row>
-    <row r="290" spans="1:22">
+    <row r="290" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A290" s="15" t="s">
         <v>24</v>
       </c>
@@ -27364,7 +27334,7 @@
       <c r="U290" s="19"/>
       <c r="V290" s="19"/>
     </row>
-    <row r="291" spans="1:22">
+    <row r="291" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A291" s="15" t="s">
         <v>24</v>
       </c>
@@ -27422,7 +27392,7 @@
       <c r="U291" s="19"/>
       <c r="V291" s="19"/>
     </row>
-    <row r="292" spans="1:22">
+    <row r="292" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A292" s="15" t="s">
         <v>24</v>
       </c>
@@ -27478,7 +27448,7 @@
       <c r="U292" s="19"/>
       <c r="V292" s="19"/>
     </row>
-    <row r="293" spans="1:22">
+    <row r="293" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A293" s="15" t="s">
         <v>24</v>
       </c>
@@ -27528,7 +27498,7 @@
       <c r="U293" s="19"/>
       <c r="V293" s="19"/>
     </row>
-    <row r="294" spans="1:22">
+    <row r="294" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A294" s="15" t="s">
         <v>24</v>
       </c>
@@ -27580,7 +27550,7 @@
       <c r="U294" s="19"/>
       <c r="V294" s="19"/>
     </row>
-    <row r="295" spans="1:22">
+    <row r="295" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A295" s="15" t="s">
         <v>194</v>
       </c>
@@ -27632,7 +27602,7 @@
       <c r="U295" s="19"/>
       <c r="V295" s="19"/>
     </row>
-    <row r="296" spans="1:22">
+    <row r="296" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A296" s="15" t="s">
         <v>78</v>
       </c>
@@ -27684,7 +27654,7 @@
       <c r="U296" s="19"/>
       <c r="V296" s="19"/>
     </row>
-    <row r="297" spans="1:22">
+    <row r="297" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A297" s="15" t="s">
         <v>24</v>
       </c>
@@ -27740,7 +27710,7 @@
       <c r="U297" s="19"/>
       <c r="V297" s="19"/>
     </row>
-    <row r="298" spans="1:22">
+    <row r="298" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A298" s="15" t="s">
         <v>24</v>
       </c>
@@ -27792,7 +27762,7 @@
       <c r="U298" s="19"/>
       <c r="V298" s="19"/>
     </row>
-    <row r="299" spans="1:22">
+    <row r="299" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A299" s="15" t="s">
         <v>24</v>
       </c>
@@ -27844,7 +27814,7 @@
       <c r="U299" s="19"/>
       <c r="V299" s="19"/>
     </row>
-    <row r="300" spans="1:22">
+    <row r="300" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A300" s="15" t="s">
         <v>476</v>
       </c>
@@ -27872,7 +27842,7 @@
       <c r="K300" s="18" t="s">
         <v>477</v>
       </c>
-      <c r="L300" s="28" t="s">
+      <c r="L300" s="26" t="s">
         <v>92</v>
       </c>
       <c r="M300" s="18"/>
@@ -27890,7 +27860,7 @@
       <c r="U300" s="19"/>
       <c r="V300" s="19"/>
     </row>
-    <row r="301" spans="1:22">
+    <row r="301" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A301" s="15" t="s">
         <v>24</v>
       </c>
@@ -27942,7 +27912,7 @@
       <c r="U301" s="19"/>
       <c r="V301" s="19"/>
     </row>
-    <row r="302" spans="1:22">
+    <row r="302" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A302" s="15" t="s">
         <v>24</v>
       </c>
@@ -27988,7 +27958,7 @@
       <c r="U302" s="19"/>
       <c r="V302" s="19"/>
     </row>
-    <row r="303" spans="1:22">
+    <row r="303" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A303" s="15" t="s">
         <v>476</v>
       </c>
@@ -28042,7 +28012,7 @@
       <c r="U303" s="19"/>
       <c r="V303" s="19"/>
     </row>
-    <row r="304" spans="1:22">
+    <row r="304" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A304" s="15" t="s">
         <v>24</v>
       </c>
@@ -28096,7 +28066,7 @@
       <c r="U304" s="19"/>
       <c r="V304" s="19"/>
     </row>
-    <row r="305" spans="1:24">
+    <row r="305" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A305" s="15" t="s">
         <v>24</v>
       </c>
@@ -28156,7 +28126,7 @@
       <c r="U305" s="19"/>
       <c r="V305" s="19"/>
     </row>
-    <row r="306" spans="1:24">
+    <row r="306" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A306" s="15" t="s">
         <v>24</v>
       </c>
@@ -28212,7 +28182,7 @@
       <c r="U306" s="19"/>
       <c r="V306" s="19"/>
     </row>
-    <row r="307" spans="1:24">
+    <row r="307" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A307" s="15" t="s">
         <v>24</v>
       </c>
@@ -28272,7 +28242,7 @@
       <c r="U307" s="19"/>
       <c r="V307" s="19"/>
     </row>
-    <row r="308" spans="1:24">
+    <row r="308" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A308" s="15" t="s">
         <v>24</v>
       </c>
@@ -28326,7 +28296,7 @@
       <c r="U308" s="19"/>
       <c r="V308" s="19"/>
     </row>
-    <row r="309" spans="1:24">
+    <row r="309" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A309" s="15" t="s">
         <v>24</v>
       </c>
@@ -28380,7 +28350,7 @@
       <c r="U309" s="19"/>
       <c r="V309" s="19"/>
     </row>
-    <row r="310" spans="1:24">
+    <row r="310" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A310" s="15" t="s">
         <v>37</v>
       </c>
@@ -28444,26 +28414,26 @@
         <v>280</v>
       </c>
     </row>
-    <row r="311" spans="1:24">
+    <row r="311" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A311" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B311" s="25">
+      <c r="B311" s="16">
         <v>46134</v>
       </c>
       <c r="C311" s="17">
         <v>0.71805555555555556</v>
       </c>
-      <c r="D311" s="25">
+      <c r="D311" s="16">
         <v>46165</v>
       </c>
       <c r="E311" s="17">
         <v>0.38055555555555554</v>
       </c>
-      <c r="F311" s="25">
+      <c r="F311" s="16">
         <v>46135</v>
       </c>
-      <c r="G311" s="25">
+      <c r="G311" s="16">
         <v>46165</v>
       </c>
       <c r="H311" s="18" t="s">
@@ -28490,13 +28460,13 @@
       <c r="O311" s="18" t="s">
         <v>506</v>
       </c>
-      <c r="P311" s="32" t="s">
+      <c r="P311" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="Q311" s="32" t="s">
+      <c r="Q311" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="R311" s="32" t="s">
+      <c r="R311" s="30" t="s">
         <v>169</v>
       </c>
       <c r="S311" s="18"/>
@@ -28516,24 +28486,24 @@
         <v>187</v>
       </c>
     </row>
-    <row r="312" spans="1:24">
+    <row r="312" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A312" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B312" s="25">
+      <c r="B312" s="16">
         <v>46135</v>
       </c>
       <c r="C312" s="17">
         <v>0.7006944444444444</v>
       </c>
-      <c r="D312" s="25">
+      <c r="D312" s="16">
         <v>46137</v>
       </c>
       <c r="E312" s="17">
         <v>0.31180555555555556</v>
       </c>
-      <c r="F312" s="25"/>
-      <c r="G312" s="25"/>
+      <c r="F312" s="16"/>
+      <c r="G312" s="16"/>
       <c r="H312" s="18" t="s">
         <v>509</v>
       </c>
@@ -28568,26 +28538,26 @@
       <c r="U312" s="19"/>
       <c r="V312" s="19"/>
     </row>
-    <row r="313" spans="1:24">
+    <row r="313" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A313" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B313" s="25">
+      <c r="B313" s="16">
         <v>46135</v>
       </c>
       <c r="C313" s="17">
         <v>0.35972222222222222</v>
       </c>
-      <c r="D313" s="25">
+      <c r="D313" s="16">
         <v>46135</v>
       </c>
       <c r="E313" s="17">
         <v>0.37986111111111109</v>
       </c>
-      <c r="F313" s="25">
+      <c r="F313" s="16">
         <v>46135</v>
       </c>
-      <c r="G313" s="25">
+      <c r="G313" s="16">
         <v>46136</v>
       </c>
       <c r="H313" s="18" t="s">
@@ -28640,26 +28610,26 @@
         <v>280</v>
       </c>
     </row>
-    <row r="314" spans="1:24">
+    <row r="314" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A314" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B314" s="25">
+      <c r="B314" s="16">
         <v>46135</v>
       </c>
       <c r="C314" s="17">
         <v>0.46180555555555558</v>
       </c>
-      <c r="D314" s="25">
+      <c r="D314" s="16">
         <v>46135</v>
       </c>
       <c r="E314" s="17">
         <v>0.55277777777777781</v>
       </c>
-      <c r="F314" s="25">
+      <c r="F314" s="16">
         <v>46140</v>
       </c>
-      <c r="G314" s="25"/>
+      <c r="G314" s="16"/>
       <c r="H314" s="18" t="s">
         <v>517</v>
       </c>
@@ -28698,24 +28668,24 @@
       <c r="U314" s="19"/>
       <c r="V314" s="19"/>
     </row>
-    <row r="315" spans="1:24">
+    <row r="315" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A315" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B315" s="25">
+      <c r="B315" s="16">
         <v>46135</v>
       </c>
       <c r="C315" s="17">
         <v>0.61875000000000002</v>
       </c>
-      <c r="D315" s="25">
+      <c r="D315" s="16">
         <v>46137</v>
       </c>
       <c r="E315" s="17">
         <v>0.32013888888888886</v>
       </c>
-      <c r="F315" s="25"/>
-      <c r="G315" s="25"/>
+      <c r="F315" s="16"/>
+      <c r="G315" s="16"/>
       <c r="H315" s="18" t="s">
         <v>63</v>
       </c>
@@ -28744,24 +28714,24 @@
       <c r="U315" s="19"/>
       <c r="V315" s="19"/>
     </row>
-    <row r="316" spans="1:24">
+    <row r="316" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A316" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B316" s="25">
+      <c r="B316" s="16">
         <v>46135</v>
       </c>
       <c r="C316" s="17">
         <v>0.58819444444444446</v>
       </c>
-      <c r="D316" s="25">
+      <c r="D316" s="16">
         <v>46135</v>
       </c>
       <c r="E316" s="17">
         <v>0.58888888888888891</v>
       </c>
-      <c r="F316" s="25"/>
-      <c r="G316" s="25"/>
+      <c r="F316" s="16"/>
+      <c r="G316" s="16"/>
       <c r="H316" s="18" t="s">
         <v>63</v>
       </c>
@@ -28794,24 +28764,24 @@
       <c r="U316" s="19"/>
       <c r="V316" s="19"/>
     </row>
-    <row r="317" spans="1:24">
+    <row r="317" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A317" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B317" s="25">
+      <c r="B317" s="16">
         <v>46135</v>
       </c>
       <c r="C317" s="17">
         <v>0.36666666666666664</v>
       </c>
-      <c r="D317" s="25">
+      <c r="D317" s="16">
         <v>46135</v>
       </c>
       <c r="E317" s="17">
         <v>0.37986111111111109</v>
       </c>
-      <c r="F317" s="25"/>
-      <c r="G317" s="25"/>
+      <c r="F317" s="16"/>
+      <c r="G317" s="16"/>
       <c r="H317" s="18" t="s">
         <v>63</v>
       </c>
@@ -28844,24 +28814,24 @@
       <c r="U317" s="19"/>
       <c r="V317" s="19"/>
     </row>
-    <row r="318" spans="1:24">
+    <row r="318" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A318" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B318" s="25">
+      <c r="B318" s="16">
         <v>46135</v>
       </c>
       <c r="C318" s="17">
         <v>0.60277777777777775</v>
       </c>
-      <c r="D318" s="25">
+      <c r="D318" s="16">
         <v>46137</v>
       </c>
       <c r="E318" s="17">
         <v>0.32569444444444445</v>
       </c>
-      <c r="F318" s="25"/>
-      <c r="G318" s="25"/>
+      <c r="F318" s="16"/>
+      <c r="G318" s="16"/>
       <c r="H318" s="18" t="s">
         <v>61</v>
       </c>
@@ -28892,26 +28862,26 @@
       <c r="U318" s="19"/>
       <c r="V318" s="19"/>
     </row>
-    <row r="319" spans="1:24">
+    <row r="319" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A319" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B319" s="25">
+      <c r="B319" s="16">
         <v>46136</v>
       </c>
       <c r="C319" s="17">
         <v>0.67361111111111116</v>
       </c>
-      <c r="D319" s="25">
+      <c r="D319" s="16">
         <v>46136</v>
       </c>
       <c r="E319" s="17">
         <v>0.67500000000000004</v>
       </c>
-      <c r="F319" s="25">
+      <c r="F319" s="16">
         <v>46137</v>
       </c>
-      <c r="G319" s="25"/>
+      <c r="G319" s="16"/>
       <c r="H319" s="18" t="s">
         <v>527</v>
       </c>
@@ -28963,26 +28933,26 @@
         <v>280</v>
       </c>
     </row>
-    <row r="320" spans="1:24">
+    <row r="320" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A320" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B320" s="25">
+      <c r="B320" s="16">
         <v>46136</v>
       </c>
       <c r="C320" s="17">
         <v>0.38541666666666669</v>
       </c>
-      <c r="D320" s="25">
+      <c r="D320" s="16">
         <v>46136</v>
       </c>
       <c r="E320" s="17">
         <v>0.38958333333333334</v>
       </c>
-      <c r="F320" s="25">
+      <c r="F320" s="16">
         <v>46136</v>
       </c>
-      <c r="G320" s="25">
+      <c r="G320" s="16">
         <v>46139</v>
       </c>
       <c r="H320" s="18" t="s">
@@ -29035,24 +29005,24 @@
         <v>280</v>
       </c>
     </row>
-    <row r="321" spans="1:22">
+    <row r="321" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A321" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B321" s="25">
+      <c r="B321" s="16">
         <v>46136</v>
       </c>
       <c r="C321" s="17">
         <v>0.66597222222222219</v>
       </c>
-      <c r="D321" s="25">
+      <c r="D321" s="16">
         <v>46137</v>
       </c>
       <c r="E321" s="17">
         <v>0.29375000000000001</v>
       </c>
-      <c r="F321" s="25"/>
-      <c r="G321" s="25"/>
+      <c r="F321" s="16"/>
+      <c r="G321" s="16"/>
       <c r="H321" s="18" t="s">
         <v>536</v>
       </c>
@@ -29085,24 +29055,24 @@
       <c r="U321" s="19"/>
       <c r="V321" s="19"/>
     </row>
-    <row r="322" spans="1:22">
+    <row r="322" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A322" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B322" s="25">
+      <c r="B322" s="16">
         <v>46136</v>
       </c>
       <c r="C322" s="17">
         <v>0.37361111111111112</v>
       </c>
-      <c r="D322" s="25">
+      <c r="D322" s="16">
         <v>46137</v>
       </c>
       <c r="E322" s="17">
         <v>0.31527777777777777</v>
       </c>
-      <c r="F322" s="25"/>
-      <c r="G322" s="25"/>
+      <c r="F322" s="16"/>
+      <c r="G322" s="16"/>
       <c r="H322" s="18" t="s">
         <v>538</v>
       </c>
@@ -29133,24 +29103,24 @@
       <c r="U322" s="19"/>
       <c r="V322" s="19"/>
     </row>
-    <row r="323" spans="1:22">
+    <row r="323" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A323" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B323" s="25">
+      <c r="B323" s="16">
         <v>46137</v>
       </c>
-      <c r="C323" s="27">
+      <c r="C323" s="25">
         <v>0.77916666666666667</v>
       </c>
-      <c r="D323" s="25">
+      <c r="D323" s="16">
         <v>46139</v>
       </c>
-      <c r="E323" s="27">
+      <c r="E323" s="25">
         <v>0.37569444444444444</v>
       </c>
-      <c r="F323" s="25"/>
-      <c r="G323" s="25"/>
+      <c r="F323" s="16"/>
+      <c r="G323" s="16"/>
       <c r="H323" s="18" t="s">
         <v>540</v>
       </c>
@@ -29163,7 +29133,7 @@
       <c r="K323" s="18">
         <v>3182527295</v>
       </c>
-      <c r="L323" s="28" t="s">
+      <c r="L323" s="26" t="s">
         <v>45</v>
       </c>
       <c r="M323" s="18" t="s">
@@ -29189,24 +29159,24 @@
       <c r="U323" s="19"/>
       <c r="V323" s="19"/>
     </row>
-    <row r="324" spans="1:22">
+    <row r="324" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A324" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B324" s="25">
+      <c r="B324" s="16">
         <v>46139</v>
       </c>
       <c r="C324" s="17">
         <v>0.36041666666666666</v>
       </c>
-      <c r="D324" s="25">
+      <c r="D324" s="16">
         <v>46139</v>
       </c>
       <c r="E324" s="17">
         <v>0.36736111111111114</v>
       </c>
-      <c r="F324" s="25"/>
-      <c r="G324" s="25"/>
+      <c r="F324" s="16"/>
+      <c r="G324" s="16"/>
       <c r="H324" s="18" t="s">
         <v>542</v>
       </c>
@@ -29243,24 +29213,24 @@
         <v>543</v>
       </c>
     </row>
-    <row r="325" spans="1:22">
+    <row r="325" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A325" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B325" s="25">
+      <c r="B325" s="16">
         <v>46139</v>
       </c>
       <c r="C325" s="17">
         <v>0.5</v>
       </c>
-      <c r="D325" s="30">
+      <c r="D325" s="28">
         <v>46139</v>
       </c>
       <c r="E325" s="17">
         <v>0.57777777777777772</v>
       </c>
-      <c r="F325" s="25"/>
-      <c r="G325" s="25"/>
+      <c r="F325" s="16"/>
+      <c r="G325" s="16"/>
       <c r="H325" s="18" t="s">
         <v>544</v>
       </c>
@@ -29301,24 +29271,24 @@
         <v>547</v>
       </c>
     </row>
-    <row r="326" spans="1:22">
+    <row r="326" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A326" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B326" s="25">
+      <c r="B326" s="16">
         <v>46139</v>
       </c>
       <c r="C326" s="17">
         <v>0.48749999999999999</v>
       </c>
-      <c r="D326" s="30">
+      <c r="D326" s="28">
         <v>46139</v>
       </c>
       <c r="E326" s="17">
         <v>0.58472222222222225</v>
       </c>
-      <c r="F326" s="25"/>
-      <c r="G326" s="25"/>
+      <c r="F326" s="16"/>
+      <c r="G326" s="16"/>
       <c r="H326" s="18" t="s">
         <v>548</v>
       </c>
@@ -29357,24 +29327,24 @@
         <v>102</v>
       </c>
     </row>
-    <row r="327" spans="1:22">
+    <row r="327" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A327" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B327" s="25">
+      <c r="B327" s="16">
         <v>46139</v>
       </c>
       <c r="C327" s="17">
         <v>0.67013888888888884</v>
       </c>
-      <c r="D327" s="25">
+      <c r="D327" s="16">
         <v>46139</v>
       </c>
       <c r="E327" s="17">
         <v>0.70208333333333328</v>
       </c>
-      <c r="F327" s="25"/>
-      <c r="G327" s="25"/>
+      <c r="F327" s="16"/>
+      <c r="G327" s="16"/>
       <c r="H327" s="18" t="s">
         <v>63</v>
       </c>
@@ -29415,24 +29385,24 @@
         <v>102</v>
       </c>
     </row>
-    <row r="328" spans="1:22">
+    <row r="328" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A328" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B328" s="25">
+      <c r="B328" s="16">
         <v>46139</v>
       </c>
       <c r="C328" s="17">
         <v>0.47499999999999998</v>
       </c>
-      <c r="D328" s="25">
+      <c r="D328" s="16">
         <v>46139</v>
       </c>
       <c r="E328" s="17">
         <v>0.58472222222222225</v>
       </c>
-      <c r="F328" s="25"/>
-      <c r="G328" s="25"/>
+      <c r="F328" s="16"/>
+      <c r="G328" s="16"/>
       <c r="H328" s="18" t="s">
         <v>63</v>
       </c>
@@ -29471,24 +29441,24 @@
       <c r="U328" s="19"/>
       <c r="V328" s="19"/>
     </row>
-    <row r="329" spans="1:22">
+    <row r="329" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A329" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B329" s="25">
+      <c r="B329" s="16">
         <v>46139</v>
       </c>
       <c r="C329" s="17">
         <v>0.48333333333333334</v>
       </c>
-      <c r="D329" s="25">
+      <c r="D329" s="16">
         <v>46139</v>
       </c>
       <c r="E329" s="17">
         <v>0.71666666666666667</v>
       </c>
-      <c r="F329" s="25"/>
-      <c r="G329" s="25"/>
+      <c r="F329" s="16"/>
+      <c r="G329" s="16"/>
       <c r="H329" s="18" t="s">
         <v>63</v>
       </c>
@@ -29527,24 +29497,24 @@
       <c r="U329" s="19"/>
       <c r="V329" s="19"/>
     </row>
-    <row r="330" spans="1:22">
+    <row r="330" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A330" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B330" s="25">
+      <c r="B330" s="16">
         <v>46139</v>
       </c>
       <c r="C330" s="17">
         <v>0.45694444444444443</v>
       </c>
-      <c r="D330" s="25">
+      <c r="D330" s="16">
         <v>46139</v>
       </c>
       <c r="E330" s="17">
         <v>0.71944444444444444</v>
       </c>
-      <c r="F330" s="25"/>
-      <c r="G330" s="25"/>
+      <c r="F330" s="16"/>
+      <c r="G330" s="16"/>
       <c r="H330" s="18" t="s">
         <v>557</v>
       </c>
@@ -29579,24 +29549,24 @@
       <c r="U330" s="19"/>
       <c r="V330" s="19"/>
     </row>
-    <row r="331" spans="1:22">
+    <row r="331" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A331" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B331" s="25">
+      <c r="B331" s="16">
         <v>46139</v>
       </c>
       <c r="C331" s="17">
         <v>0.87013888888888891</v>
       </c>
-      <c r="D331" s="25">
+      <c r="D331" s="16">
         <v>46140</v>
       </c>
       <c r="E331" s="17">
         <v>0.34652777777777777</v>
       </c>
-      <c r="F331" s="25"/>
-      <c r="G331" s="25"/>
+      <c r="F331" s="16"/>
+      <c r="G331" s="16"/>
       <c r="H331" s="18" t="s">
         <v>63</v>
       </c>
@@ -29635,24 +29605,24 @@
       <c r="U331" s="19"/>
       <c r="V331" s="19"/>
     </row>
-    <row r="332" spans="1:22">
+    <row r="332" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A332" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="B332" s="25">
+      <c r="B332" s="16">
         <v>46140</v>
       </c>
       <c r="C332" s="17">
         <v>0.30972222222222223</v>
       </c>
-      <c r="D332" s="25">
+      <c r="D332" s="16">
         <v>46140</v>
       </c>
       <c r="E332" s="17">
         <v>0.34722222222222221</v>
       </c>
-      <c r="F332" s="25"/>
-      <c r="G332" s="25"/>
+      <c r="F332" s="16"/>
+      <c r="G332" s="16"/>
       <c r="H332" s="10" t="s">
         <v>563</v>
       </c>
@@ -29689,24 +29659,24 @@
       <c r="U332" s="19"/>
       <c r="V332" s="19"/>
     </row>
-    <row r="333" spans="1:22">
+    <row r="333" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A333" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B333" s="25">
+      <c r="B333" s="16">
         <v>46140</v>
       </c>
       <c r="C333" s="17">
         <v>0.53055555555555556</v>
       </c>
-      <c r="D333" s="25">
+      <c r="D333" s="16">
         <v>46140</v>
       </c>
       <c r="E333" s="17">
         <v>0.53055555555555556</v>
       </c>
-      <c r="F333" s="25"/>
-      <c r="G333" s="25"/>
+      <c r="F333" s="16"/>
+      <c r="G333" s="16"/>
       <c r="H333" s="18" t="s">
         <v>61</v>
       </c>
@@ -29741,24 +29711,24 @@
       <c r="U333" s="19"/>
       <c r="V333" s="19"/>
     </row>
-    <row r="334" spans="1:22">
+    <row r="334" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A334" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B334" s="25">
+      <c r="B334" s="16">
         <v>46140</v>
       </c>
       <c r="C334" s="17">
         <v>0.45277777777777778</v>
       </c>
-      <c r="D334" s="25">
+      <c r="D334" s="16">
         <v>46140</v>
       </c>
       <c r="E334" s="17">
         <v>0.68402777777777779</v>
       </c>
-      <c r="F334" s="25"/>
-      <c r="G334" s="25"/>
+      <c r="F334" s="16"/>
+      <c r="G334" s="16"/>
       <c r="H334" s="18" t="s">
         <v>567</v>
       </c>
@@ -29797,24 +29767,24 @@
       <c r="U334" s="19"/>
       <c r="V334" s="19"/>
     </row>
-    <row r="335" spans="1:22">
+    <row r="335" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A335" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B335" s="25">
+      <c r="B335" s="16">
         <v>46140</v>
       </c>
       <c r="C335" s="17">
         <v>0.4465277777777778</v>
       </c>
-      <c r="D335" s="25">
+      <c r="D335" s="16">
         <v>46140</v>
       </c>
       <c r="E335" s="17">
         <v>0.68680555555555556</v>
       </c>
-      <c r="F335" s="25"/>
-      <c r="G335" s="25"/>
+      <c r="F335" s="16"/>
+      <c r="G335" s="16"/>
       <c r="H335" s="18" t="s">
         <v>61</v>
       </c>
@@ -29853,24 +29823,24 @@
       <c r="U335" s="19"/>
       <c r="V335" s="19"/>
     </row>
-    <row r="336" spans="1:22">
+    <row r="336" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A336" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B336" s="25">
+      <c r="B336" s="16">
         <v>46140</v>
       </c>
       <c r="C336" s="17">
         <v>0.42291666666666666</v>
       </c>
-      <c r="D336" s="25">
+      <c r="D336" s="16">
         <v>46140</v>
       </c>
       <c r="E336" s="17">
         <v>0.42430555555555555</v>
       </c>
-      <c r="F336" s="25"/>
-      <c r="G336" s="25"/>
+      <c r="F336" s="16"/>
+      <c r="G336" s="16"/>
       <c r="H336" s="18" t="s">
         <v>571</v>
       </c>
@@ -29909,24 +29879,24 @@
       <c r="U336" s="19"/>
       <c r="V336" s="19"/>
     </row>
-    <row r="337" spans="1:24">
+    <row r="337" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A337" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B337" s="25">
+      <c r="B337" s="16">
         <v>46138</v>
       </c>
       <c r="C337" s="17">
         <v>0.80763888888888891</v>
       </c>
-      <c r="D337" s="25">
+      <c r="D337" s="16">
         <v>46140</v>
       </c>
       <c r="E337" s="17">
         <v>0.37222222222222223</v>
       </c>
-      <c r="F337" s="25"/>
-      <c r="G337" s="25"/>
+      <c r="F337" s="16"/>
+      <c r="G337" s="16"/>
       <c r="H337" s="18" t="s">
         <v>571</v>
       </c>
@@ -29965,24 +29935,24 @@
       <c r="U337" s="19"/>
       <c r="V337" s="19"/>
     </row>
-    <row r="338" spans="1:24">
+    <row r="338" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A338" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B338" s="25">
+      <c r="B338" s="16">
         <v>46139</v>
       </c>
       <c r="C338" s="17">
         <v>0.31805555555555554</v>
       </c>
-      <c r="D338" s="25">
+      <c r="D338" s="16">
         <v>46139</v>
       </c>
       <c r="E338" s="17">
         <v>0.37152777777777779</v>
       </c>
-      <c r="F338" s="25"/>
-      <c r="G338" s="25"/>
+      <c r="F338" s="16"/>
+      <c r="G338" s="16"/>
       <c r="H338" s="18" t="s">
         <v>576</v>
       </c>
@@ -30021,24 +29991,24 @@
       <c r="U338" s="19"/>
       <c r="V338" s="19"/>
     </row>
-    <row r="339" spans="1:24">
+    <row r="339" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A339" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B339" s="25">
+      <c r="B339" s="16">
         <v>46141</v>
       </c>
       <c r="C339" s="17">
         <v>0.40347222222222223</v>
       </c>
-      <c r="D339" s="25">
+      <c r="D339" s="16">
         <v>46141</v>
       </c>
       <c r="E339" s="17">
         <v>0.41388888888888886</v>
       </c>
-      <c r="F339" s="25"/>
-      <c r="G339" s="25"/>
+      <c r="F339" s="16"/>
+      <c r="G339" s="16"/>
       <c r="H339" s="18" t="s">
         <v>63</v>
       </c>
@@ -30081,24 +30051,24 @@
         <v>582</v>
       </c>
     </row>
-    <row r="340" spans="1:24">
+    <row r="340" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A340" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B340" s="25">
+      <c r="B340" s="16">
         <v>46141</v>
       </c>
       <c r="C340" s="17">
         <v>0.41666666666666669</v>
       </c>
-      <c r="D340" s="25">
+      <c r="D340" s="16">
         <v>46141</v>
       </c>
       <c r="E340" s="17">
         <v>0.41944444444444445</v>
       </c>
-      <c r="F340" s="25"/>
-      <c r="G340" s="25"/>
+      <c r="F340" s="16"/>
+      <c r="G340" s="16"/>
       <c r="H340" s="18" t="s">
         <v>583</v>
       </c>
@@ -30137,24 +30107,24 @@
       <c r="U340" s="19"/>
       <c r="V340" s="19"/>
     </row>
-    <row r="341" spans="1:24">
+    <row r="341" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A341" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B341" s="25">
+      <c r="B341" s="16">
         <v>46141</v>
       </c>
       <c r="C341" s="17">
         <v>0.44513888888888886</v>
       </c>
-      <c r="D341" s="25">
+      <c r="D341" s="16">
         <v>46141</v>
       </c>
       <c r="E341" s="17">
         <v>0.47916666666666669</v>
       </c>
-      <c r="F341" s="25"/>
-      <c r="G341" s="25"/>
+      <c r="F341" s="16"/>
+      <c r="G341" s="16"/>
       <c r="H341" s="18" t="s">
         <v>585</v>
       </c>
@@ -30195,63 +30165,61 @@
       <c r="U341" s="19"/>
       <c r="V341" s="19"/>
     </row>
-    <row r="342" spans="1:24">
-      <c r="A342" s="35" t="s">
+    <row r="342" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A342" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="B342" s="25">
+      <c r="B342" s="16">
         <v>46139</v>
       </c>
-      <c r="C342" s="37">
+      <c r="C342" s="17">
         <v>0.46458333333333335</v>
       </c>
-      <c r="D342" s="25">
+      <c r="D342" s="16">
         <v>46139</v>
       </c>
-      <c r="E342" s="37">
+      <c r="E342" s="17">
         <v>0.46458333333333335</v>
       </c>
-      <c r="F342" s="36"/>
-      <c r="G342" s="36"/>
-      <c r="H342" s="33" t="s">
+      <c r="F342" s="16"/>
+      <c r="G342" s="16"/>
+      <c r="H342" s="18" t="s">
         <v>589</v>
       </c>
-      <c r="I342" s="33" t="s">
+      <c r="I342" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="J342" s="33" t="s">
+      <c r="J342" s="18" t="s">
         <v>590</v>
       </c>
-      <c r="K342" s="33" t="s">
+      <c r="K342" s="18" t="s">
         <v>591</v>
       </c>
-      <c r="L342" s="33" t="s">
+      <c r="L342" s="18" t="s">
         <v>27</v>
       </c>
       <c r="M342" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="N342" s="33" t="s">
+      <c r="N342" s="18" t="s">
         <v>515</v>
       </c>
-      <c r="O342" s="33" t="s">
+      <c r="O342" s="18" t="s">
         <v>455</v>
       </c>
-      <c r="P342" s="33" t="s">
+      <c r="P342" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="Q342" s="33" t="s">
+      <c r="Q342" s="18" t="s">
         <v>116</v>
       </c>
       <c r="R342" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="S342" s="33"/>
-      <c r="T342" s="33"/>
-      <c r="U342" s="34"/>
-      <c r="V342" s="34"/>
-      <c r="W342" s="38"/>
-      <c r="X342" s="38"/>
+      <c r="S342" s="18"/>
+      <c r="T342" s="18"/>
+      <c r="U342" s="19"/>
+      <c r="V342" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -30305,7 +30273,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0665A305-334F-4716-9D07-6A8B74E7F902}">
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.5703125" bestFit="1" customWidth="1"/>
@@ -30319,7 +30287,7 @@
     <col min="17" max="17" width="20.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -30351,7 +30319,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>35</v>
       </c>
@@ -30383,7 +30351,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>28</v>
       </c>
@@ -30415,7 +30383,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>73</v>
       </c>
@@ -30447,7 +30415,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>66</v>
       </c>
@@ -30470,7 +30438,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>605</v>
       </c>
@@ -30493,7 +30461,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>130</v>
       </c>
@@ -30516,7 +30484,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>56</v>
       </c>
@@ -30536,7 +30504,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>201</v>
       </c>
@@ -30559,7 +30527,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>90</v>
       </c>
@@ -30576,7 +30544,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>618</v>
       </c>
@@ -30590,7 +30558,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>220</v>
       </c>
@@ -30601,7 +30569,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>623</v>
       </c>
@@ -30609,7 +30577,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>624</v>
       </c>
@@ -30617,7 +30585,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>625</v>
       </c>
@@ -30625,42 +30593,42 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>626</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="18" spans="1:1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:1">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:1">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -30683,7 +30651,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB659A03-ECAA-4F5A-8B42-DE82986E8B1D}">
   <dimension ref="A1:D76"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -30794,7 +30762,7 @@
     <col min="110" max="110" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>16</v>
       </c>
@@ -30802,7 +30770,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
         <v>7</v>
       </c>
@@ -30816,7 +30784,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -30830,22 +30798,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>628</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>630</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>235</v>
       </c>
@@ -30859,22 +30827,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>631</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>632</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>633</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>226</v>
       </c>
@@ -30888,22 +30856,22 @@
         <v>169</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>634</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>283</v>
       </c>
@@ -30917,22 +30885,22 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
         <v>636</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>206</v>
       </c>
@@ -30946,22 +30914,22 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>639</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>632</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>640</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -30975,22 +30943,22 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
         <v>641</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -31004,22 +30972,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C29" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>159</v>
       </c>
@@ -31033,22 +31001,22 @@
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
         <v>628</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>645</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>219</v>
       </c>
@@ -31062,22 +31030,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C37" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>292</v>
       </c>
@@ -31091,22 +31059,22 @@
         <v>293</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C41" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>650</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>156</v>
       </c>
@@ -31120,22 +31088,22 @@
         <v>57</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C45" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>632</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>652</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>228</v>
       </c>
@@ -31149,22 +31117,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C49" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>653</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>182</v>
       </c>
@@ -31178,22 +31146,22 @@
         <v>183</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C53" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>655</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>179</v>
       </c>
@@ -31207,22 +31175,22 @@
         <v>112</v>
       </c>
     </row>
-    <row r="57" spans="1:4">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C57" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="58" spans="1:4">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>656</v>
       </c>
     </row>
-    <row r="60" spans="1:4">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>317</v>
       </c>
@@ -31236,22 +31204,22 @@
         <v>54</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C61" t="s">
         <v>636</v>
       </c>
     </row>
-    <row r="62" spans="1:4">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="63" spans="1:4">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>657</v>
       </c>
     </row>
-    <row r="64" spans="1:4">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>291</v>
       </c>
@@ -31265,22 +31233,22 @@
         <v>169</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="66" spans="1:4">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="67" spans="1:4">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>167</v>
       </c>
@@ -31294,22 +31262,22 @@
         <v>169</v>
       </c>
     </row>
-    <row r="69" spans="1:4">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C69" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="70" spans="1:4">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="71" spans="1:4">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>659</v>
       </c>
     </row>
-    <row r="72" spans="1:4">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>111</v>
       </c>
@@ -31323,22 +31291,22 @@
         <v>112</v>
       </c>
     </row>
-    <row r="73" spans="1:4">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C73" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="74" spans="1:4">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="75" spans="1:4">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>661</v>
       </c>
     </row>
-    <row r="76" spans="1:4">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>662</v>
       </c>

</xml_diff>

<commit_message>
ajustes visuales dashboard crm operaciones
</commit_message>
<xml_diff>
--- a/BD CRM 14042026.xlsx
+++ b/BD CRM 14042026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tractocar-my.sharepoint.com/personal/avera_tractocar_com/Documents/Team Comercial/CRM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2017" documentId="8_{F2A5B7CE-E8D2-40BD-8C9A-6BB22E881C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C77EB92D-C6BB-4BEE-8667-160542669CB4}"/>
+  <xr:revisionPtr revIDLastSave="2215" documentId="8_{F2A5B7CE-E8D2-40BD-8C9A-6BB22E881C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E200359-C5C3-45D7-BD8F-E7837C1A757C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E68C7C40-B1B6-4540-8438-F3ACB83D4A52}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="915" r:id="rId4"/>
+    <pivotCache cacheId="959" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3755" uniqueCount="698">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3939" uniqueCount="729">
   <si>
     <t>Canal</t>
   </si>
@@ -1934,6 +1934,99 @@
   </si>
   <si>
     <t>311 5852286</t>
+  </si>
+  <si>
+    <t>Mayra Guerrero</t>
+  </si>
+  <si>
+    <t>318 2508054</t>
+  </si>
+  <si>
+    <t>318 8216486</t>
+  </si>
+  <si>
+    <t>323 2333896</t>
+  </si>
+  <si>
+    <t>Fibra Andina</t>
+  </si>
+  <si>
+    <t>Lina Vargas</t>
+  </si>
+  <si>
+    <t>304 5872151</t>
+  </si>
+  <si>
+    <t>Oficina Magda</t>
+  </si>
+  <si>
+    <t>312 4693667</t>
+  </si>
+  <si>
+    <t>301 3739878</t>
+  </si>
+  <si>
+    <t>Manuel</t>
+  </si>
+  <si>
+    <t>318 5523579</t>
+  </si>
+  <si>
+    <t>Wissam</t>
+  </si>
+  <si>
+    <t>300 2074028</t>
+  </si>
+  <si>
+    <t>Angy Acuña</t>
+  </si>
+  <si>
+    <t>301 3047613</t>
+  </si>
+  <si>
+    <t>Sencillo - Furgonado</t>
+  </si>
+  <si>
+    <t>Rocio</t>
+  </si>
+  <si>
+    <t>322 2908930</t>
+  </si>
+  <si>
+    <t>+58 414-7324901</t>
+  </si>
+  <si>
+    <t>Oscar Castro</t>
+  </si>
+  <si>
+    <t>311 7923235</t>
+  </si>
+  <si>
+    <t>Procalco</t>
+  </si>
+  <si>
+    <t>312 7120197</t>
+  </si>
+  <si>
+    <t>Lock Seal Colombia</t>
+  </si>
+  <si>
+    <t>304 4661339</t>
+  </si>
+  <si>
+    <t>Precinto</t>
+  </si>
+  <si>
+    <t>Jose Ricardo Suarez</t>
+  </si>
+  <si>
+    <t>314 8677282</t>
+  </si>
+  <si>
+    <t>CFC logistic</t>
+  </si>
+  <si>
+    <t>RODRIGO</t>
   </si>
   <si>
     <t>Comentarios</t>
@@ -3364,7 +3457,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Excel Services" refreshedDate="46133.363129745368" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="306" xr:uid="{F76DB425-280F-4732-9ABC-0DBAAE885F3C}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:W357" sheet="BD"/>
+    <worksheetSource ref="A1:W373" sheet="BD"/>
   </cacheSource>
   <cacheFields count="23">
     <cacheField name="Canal" numFmtId="0">
@@ -11285,7 +11378,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{85491199-660D-426C-9385-E7AF8A153D4E}" name="TablaDinámica1" cacheId="915" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{85491199-660D-426C-9385-E7AF8A153D4E}" name="TablaDinámica1" cacheId="959" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:D76" firstHeaderRow="1" firstDataRow="1" firstDataCol="4" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="23">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -11811,8 +11904,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3B0873A0-70FC-403E-BC89-61BBA66734E5}" name="Tabla1" displayName="Tabla1" ref="A1:X357" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28" headerRowBorderDxfId="26" tableBorderDxfId="27" totalsRowBorderDxfId="25">
-  <autoFilter ref="A1:X357" xr:uid="{3B0873A0-70FC-403E-BC89-61BBA66734E5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3B0873A0-70FC-403E-BC89-61BBA66734E5}" name="Tabla1" displayName="Tabla1" ref="A1:X373" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28" headerRowBorderDxfId="26" tableBorderDxfId="27" totalsRowBorderDxfId="25">
+  <autoFilter ref="A1:X373" xr:uid="{3B0873A0-70FC-403E-BC89-61BBA66734E5}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:X336">
     <sortCondition ref="B1:B336"/>
   </sortState>
@@ -12225,7 +12318,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C5770D-06F6-4265-B815-90352D3707BC}">
-  <dimension ref="A1:X357"/>
+  <dimension ref="A1:X373"/>
   <sheetFormatPr defaultColWidth="17.42578125" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="11" width="17.42578125" style="12"/>
@@ -27081,7 +27174,9 @@
       <c r="L283" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="M283" s="10"/>
+      <c r="M283" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="N283" s="18"/>
       <c r="O283" s="18"/>
       <c r="P283" s="18" t="s">
@@ -31089,7 +31184,7 @@
         <v>528</v>
       </c>
       <c r="I356" s="18" t="s">
-        <v>61</v>
+        <v>470</v>
       </c>
       <c r="J356" s="18" t="s">
         <v>629</v>
@@ -31098,7 +31193,7 @@
         <v>630</v>
       </c>
       <c r="L356" s="18" t="s">
-        <v>61</v>
+        <v>454</v>
       </c>
       <c r="M356" s="18" t="s">
         <v>61</v>
@@ -31143,23 +31238,929 @@
       </c>
       <c r="F357" s="38"/>
       <c r="G357" s="38"/>
-      <c r="H357" s="35"/>
-      <c r="I357" s="35"/>
-      <c r="J357" s="35"/>
-      <c r="K357" s="35"/>
-      <c r="L357" s="35"/>
-      <c r="M357" s="35"/>
-      <c r="N357" s="35"/>
-      <c r="O357" s="35"/>
-      <c r="P357" s="35"/>
-      <c r="Q357" s="35"/>
-      <c r="R357" s="35"/>
+      <c r="H357" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="I357" s="35" t="s">
+        <v>470</v>
+      </c>
+      <c r="J357" s="35" t="s">
+        <v>631</v>
+      </c>
+      <c r="K357" s="35" t="s">
+        <v>632</v>
+      </c>
+      <c r="L357" s="35" t="s">
+        <v>454</v>
+      </c>
+      <c r="M357" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="N357" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O357" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P357" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q357" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R357" s="18" t="s">
+        <v>85</v>
+      </c>
       <c r="S357" s="35"/>
       <c r="T357" s="35"/>
       <c r="U357" s="36"/>
       <c r="V357" s="36"/>
       <c r="W357" s="40"/>
       <c r="X357" s="40"/>
+    </row>
+    <row r="358" spans="1:24">
+      <c r="A358" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B358" s="38">
+        <v>46134</v>
+      </c>
+      <c r="C358" s="39">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="D358" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E358" s="39">
+        <v>0.65625</v>
+      </c>
+      <c r="F358" s="38"/>
+      <c r="G358" s="38"/>
+      <c r="H358" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="I358" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="J358" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="K358" s="35" t="s">
+        <v>633</v>
+      </c>
+      <c r="L358" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="M358" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="N358" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O358" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P358" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q358" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R358" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S358" s="35"/>
+      <c r="T358" s="35"/>
+      <c r="U358" s="36"/>
+      <c r="V358" s="36"/>
+      <c r="W358" s="40"/>
+      <c r="X358" s="40"/>
+    </row>
+    <row r="359" spans="1:24">
+      <c r="A359" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B359" s="38">
+        <v>46134</v>
+      </c>
+      <c r="C359" s="39">
+        <v>0.47222222222222221</v>
+      </c>
+      <c r="D359" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E359" s="39">
+        <v>0.65833333333333333</v>
+      </c>
+      <c r="F359" s="38"/>
+      <c r="G359" s="38"/>
+      <c r="H359" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="I359" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="J359" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="K359" s="35" t="s">
+        <v>634</v>
+      </c>
+      <c r="L359" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="M359" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="N359" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O359" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P359" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q359" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R359" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S359" s="35"/>
+      <c r="T359" s="35"/>
+      <c r="U359" s="36"/>
+      <c r="V359" s="36"/>
+      <c r="W359" s="40"/>
+      <c r="X359" s="40"/>
+    </row>
+    <row r="360" spans="1:24">
+      <c r="A360" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B360" s="38">
+        <v>46134</v>
+      </c>
+      <c r="C360" s="39">
+        <v>0.42916666666666664</v>
+      </c>
+      <c r="D360" s="38">
+        <v>46134</v>
+      </c>
+      <c r="E360" s="39">
+        <v>0.44166666666666665</v>
+      </c>
+      <c r="F360" s="38"/>
+      <c r="G360" s="38"/>
+      <c r="H360" s="35" t="s">
+        <v>635</v>
+      </c>
+      <c r="I360" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="J360" s="35" t="s">
+        <v>636</v>
+      </c>
+      <c r="K360" s="35" t="s">
+        <v>637</v>
+      </c>
+      <c r="L360" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="M360" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="N360" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O360" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P360" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q360" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R360" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S360" s="35"/>
+      <c r="T360" s="35"/>
+      <c r="U360" s="36"/>
+      <c r="V360" s="36"/>
+      <c r="W360" s="40"/>
+      <c r="X360" s="40"/>
+    </row>
+    <row r="361" spans="1:24">
+      <c r="A361" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B361" s="38">
+        <v>46134</v>
+      </c>
+      <c r="C361" s="39">
+        <v>0.43263888888888891</v>
+      </c>
+      <c r="D361" s="38">
+        <v>46134</v>
+      </c>
+      <c r="E361" s="39">
+        <v>0.43333333333333335</v>
+      </c>
+      <c r="F361" s="38"/>
+      <c r="G361" s="38"/>
+      <c r="H361" s="35" t="s">
+        <v>638</v>
+      </c>
+      <c r="I361" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="J361" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="K361" s="35" t="s">
+        <v>639</v>
+      </c>
+      <c r="L361" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="M361" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="N361" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O361" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P361" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q361" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R361" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S361" s="35"/>
+      <c r="T361" s="35"/>
+      <c r="U361" s="36"/>
+      <c r="V361" s="36"/>
+      <c r="W361" s="40"/>
+      <c r="X361" s="40"/>
+    </row>
+    <row r="362" spans="1:24">
+      <c r="A362" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B362" s="38">
+        <v>46134</v>
+      </c>
+      <c r="C362" s="39">
+        <v>0.41388888888888886</v>
+      </c>
+      <c r="D362" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E362" s="39">
+        <v>0.66319444444444442</v>
+      </c>
+      <c r="F362" s="38"/>
+      <c r="G362" s="38"/>
+      <c r="H362" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="I362" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="J362" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="K362" s="35" t="s">
+        <v>640</v>
+      </c>
+      <c r="L362" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="M362" s="35" t="s">
+        <v>101</v>
+      </c>
+      <c r="N362" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O362" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P362" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q362" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R362" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S362" s="35"/>
+      <c r="T362" s="35"/>
+      <c r="U362" s="36"/>
+      <c r="V362" s="36"/>
+      <c r="W362" s="40"/>
+      <c r="X362" s="40"/>
+    </row>
+    <row r="363" spans="1:24">
+      <c r="A363" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B363" s="38">
+        <v>46134</v>
+      </c>
+      <c r="C363" s="39">
+        <v>0.37430555555555556</v>
+      </c>
+      <c r="D363" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E363" s="39">
+        <v>0.66527777777777775</v>
+      </c>
+      <c r="F363" s="38"/>
+      <c r="G363" s="38"/>
+      <c r="H363" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="I363" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="J363" s="35" t="s">
+        <v>641</v>
+      </c>
+      <c r="K363" s="35" t="s">
+        <v>642</v>
+      </c>
+      <c r="L363" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="M363" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="N363" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O363" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P363" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q363" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R363" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S363" s="35"/>
+      <c r="T363" s="35"/>
+      <c r="U363" s="36"/>
+      <c r="V363" s="36"/>
+      <c r="W363" s="40"/>
+      <c r="X363" s="40"/>
+    </row>
+    <row r="364" spans="1:24">
+      <c r="A364" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B364" s="38">
+        <v>46133</v>
+      </c>
+      <c r="C364" s="39">
+        <v>0.80763888888888891</v>
+      </c>
+      <c r="D364" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E364" s="39">
+        <v>0.67083333333333328</v>
+      </c>
+      <c r="F364" s="38"/>
+      <c r="G364" s="38"/>
+      <c r="H364" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="I364" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="J364" s="35" t="s">
+        <v>643</v>
+      </c>
+      <c r="K364" s="35" t="s">
+        <v>644</v>
+      </c>
+      <c r="L364" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="M364" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="N364" s="35"/>
+      <c r="O364" s="35"/>
+      <c r="P364" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q364" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="R364" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S364" s="35"/>
+      <c r="T364" s="35"/>
+      <c r="U364" s="36"/>
+      <c r="V364" s="36"/>
+      <c r="W364" s="40"/>
+      <c r="X364" s="40"/>
+    </row>
+    <row r="365" spans="1:24">
+      <c r="A365" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B365" s="38">
+        <v>46133</v>
+      </c>
+      <c r="C365" s="39">
+        <v>0.71944444444444444</v>
+      </c>
+      <c r="D365" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E365" s="39">
+        <v>0.67291666666666672</v>
+      </c>
+      <c r="F365" s="38"/>
+      <c r="G365" s="38"/>
+      <c r="H365" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="I365" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="J365" s="35" t="s">
+        <v>645</v>
+      </c>
+      <c r="K365" s="35" t="s">
+        <v>646</v>
+      </c>
+      <c r="L365" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="M365" s="35" t="s">
+        <v>101</v>
+      </c>
+      <c r="N365" s="35" t="s">
+        <v>279</v>
+      </c>
+      <c r="O365" s="35" t="s">
+        <v>279</v>
+      </c>
+      <c r="P365" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q365" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R365" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="S365" s="35"/>
+      <c r="T365" s="35"/>
+      <c r="U365" s="36"/>
+      <c r="V365" s="36" t="s">
+        <v>647</v>
+      </c>
+      <c r="W365" s="40"/>
+      <c r="X365" s="40"/>
+    </row>
+    <row r="366" spans="1:24">
+      <c r="A366" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B366" s="38">
+        <v>46133</v>
+      </c>
+      <c r="C366" s="39">
+        <v>0.68611111111111112</v>
+      </c>
+      <c r="D366" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E366" s="39">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="F366" s="38"/>
+      <c r="G366" s="38"/>
+      <c r="H366" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="I366" s="35" t="s">
+        <v>470</v>
+      </c>
+      <c r="J366" s="35" t="s">
+        <v>648</v>
+      </c>
+      <c r="K366" s="35" t="s">
+        <v>649</v>
+      </c>
+      <c r="L366" s="35" t="s">
+        <v>454</v>
+      </c>
+      <c r="M366" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="N366" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O366" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P366" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q366" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R366" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S366" s="35"/>
+      <c r="T366" s="35"/>
+      <c r="U366" s="36"/>
+      <c r="V366" s="36"/>
+      <c r="W366" s="40"/>
+      <c r="X366" s="40"/>
+    </row>
+    <row r="367" spans="1:24">
+      <c r="A367" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B367" s="38">
+        <v>46133</v>
+      </c>
+      <c r="C367" s="39">
+        <v>0.68055555555555558</v>
+      </c>
+      <c r="D367" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E367" s="39">
+        <v>0.67847222222222225</v>
+      </c>
+      <c r="F367" s="38"/>
+      <c r="G367" s="38"/>
+      <c r="H367" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="I367" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="J367" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="K367" s="35" t="s">
+        <v>650</v>
+      </c>
+      <c r="L367" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="M367" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="N367" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O367" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P367" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q367" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R367" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S367" s="35"/>
+      <c r="T367" s="35"/>
+      <c r="U367" s="36"/>
+      <c r="V367" s="36"/>
+      <c r="W367" s="40"/>
+      <c r="X367" s="40"/>
+    </row>
+    <row r="368" spans="1:24">
+      <c r="A368" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B368" s="38">
+        <v>46133</v>
+      </c>
+      <c r="C368" s="39">
+        <v>0.67777777777777781</v>
+      </c>
+      <c r="D368" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E368" s="39">
+        <v>0.67986111111111114</v>
+      </c>
+      <c r="F368" s="38"/>
+      <c r="G368" s="38"/>
+      <c r="H368" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="I368" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="J368" s="35" t="s">
+        <v>651</v>
+      </c>
+      <c r="K368" s="35" t="s">
+        <v>652</v>
+      </c>
+      <c r="L368" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="M368" s="35" t="s">
+        <v>468</v>
+      </c>
+      <c r="N368" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O368" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P368" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q368" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R368" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S368" s="35"/>
+      <c r="T368" s="35"/>
+      <c r="U368" s="36"/>
+      <c r="V368" s="36"/>
+      <c r="W368" s="40"/>
+      <c r="X368" s="40"/>
+    </row>
+    <row r="369" spans="1:24">
+      <c r="A369" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B369" s="38">
+        <v>46133</v>
+      </c>
+      <c r="C369" s="39">
+        <v>0.64444444444444449</v>
+      </c>
+      <c r="D369" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E369" s="39">
+        <v>0.68263888888888891</v>
+      </c>
+      <c r="F369" s="38"/>
+      <c r="G369" s="38"/>
+      <c r="H369" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="I369" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="J369" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="K369" s="35" t="s">
+        <v>654</v>
+      </c>
+      <c r="L369" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="M369" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="N369" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O369" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P369" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q369" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R369" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S369" s="35"/>
+      <c r="T369" s="35"/>
+      <c r="U369" s="36"/>
+      <c r="V369" s="36"/>
+      <c r="W369" s="40"/>
+      <c r="X369" s="40"/>
+    </row>
+    <row r="370" spans="1:24">
+      <c r="A370" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B370" s="38">
+        <v>46133</v>
+      </c>
+      <c r="C370" s="39">
+        <v>0.62361111111111112</v>
+      </c>
+      <c r="D370" s="25">
+        <v>46142</v>
+      </c>
+      <c r="E370" s="39">
+        <v>0.68333333333333335</v>
+      </c>
+      <c r="F370" s="38"/>
+      <c r="G370" s="38"/>
+      <c r="H370" s="35" t="s">
+        <v>655</v>
+      </c>
+      <c r="I370" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="J370" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="K370" s="35" t="s">
+        <v>656</v>
+      </c>
+      <c r="L370" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="M370" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="N370" s="35" t="s">
+        <v>455</v>
+      </c>
+      <c r="O370" s="35" t="s">
+        <v>486</v>
+      </c>
+      <c r="P370" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q370" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R370" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S370" s="35"/>
+      <c r="T370" s="35"/>
+      <c r="U370" s="36"/>
+      <c r="V370" s="36" t="s">
+        <v>657</v>
+      </c>
+      <c r="W370" s="40"/>
+      <c r="X370" s="40"/>
+    </row>
+    <row r="371" spans="1:24">
+      <c r="A371" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B371" s="38">
+        <v>46133</v>
+      </c>
+      <c r="C371" s="39">
+        <v>0.50069444444444444</v>
+      </c>
+      <c r="D371" s="38">
+        <v>46142</v>
+      </c>
+      <c r="E371" s="39">
+        <v>0.69027777777777777</v>
+      </c>
+      <c r="F371" s="38"/>
+      <c r="G371" s="38"/>
+      <c r="H371" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="I371" s="35" t="s">
+        <v>470</v>
+      </c>
+      <c r="J371" s="35" t="s">
+        <v>658</v>
+      </c>
+      <c r="K371" s="35" t="s">
+        <v>659</v>
+      </c>
+      <c r="L371" s="35" t="s">
+        <v>454</v>
+      </c>
+      <c r="M371" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="N371" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O371" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="P371" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q371" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="R371" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="S371" s="35"/>
+      <c r="T371" s="35"/>
+      <c r="U371" s="36"/>
+      <c r="V371" s="36"/>
+      <c r="W371" s="40"/>
+      <c r="X371" s="40"/>
+    </row>
+    <row r="372" spans="1:24">
+      <c r="A372" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B372" s="38">
+        <v>46134</v>
+      </c>
+      <c r="C372" s="39">
+        <v>0.43055555555555558</v>
+      </c>
+      <c r="D372" s="38">
+        <v>46134</v>
+      </c>
+      <c r="E372" s="39">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="F372" s="38"/>
+      <c r="G372" s="38"/>
+      <c r="H372" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="I372" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="J372" s="35" t="s">
+        <v>661</v>
+      </c>
+      <c r="K372" s="35">
+        <v>3113050369</v>
+      </c>
+      <c r="L372" s="35"/>
+      <c r="M372" s="35"/>
+      <c r="N372" s="35"/>
+      <c r="O372" s="35"/>
+      <c r="P372" s="35"/>
+      <c r="Q372" s="35"/>
+      <c r="R372" s="35"/>
+      <c r="S372" s="35"/>
+      <c r="T372" s="35"/>
+      <c r="U372" s="36"/>
+      <c r="V372" s="36"/>
+      <c r="W372" s="40"/>
+      <c r="X372" s="40"/>
+    </row>
+    <row r="373" spans="1:24">
+      <c r="A373" s="37"/>
+      <c r="B373" s="38"/>
+      <c r="C373" s="39"/>
+      <c r="D373" s="38"/>
+      <c r="E373" s="39"/>
+      <c r="F373" s="38"/>
+      <c r="G373" s="38"/>
+      <c r="H373" s="35"/>
+      <c r="I373" s="35"/>
+      <c r="J373" s="35"/>
+      <c r="K373" s="35">
+        <v>3154088613</v>
+      </c>
+      <c r="L373" s="35"/>
+      <c r="M373" s="35"/>
+      <c r="N373" s="35"/>
+      <c r="O373" s="35"/>
+      <c r="P373" s="35"/>
+      <c r="Q373" s="35"/>
+      <c r="R373" s="35"/>
+      <c r="S373" s="35"/>
+      <c r="T373" s="35"/>
+      <c r="U373" s="36"/>
+      <c r="V373" s="36"/>
+      <c r="W373" s="40"/>
+      <c r="X373" s="40"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31208,7 +32209,7 @@
           <x14:formula1>
             <xm:f>Glosario!$F$2:$F$10</xm:f>
           </x14:formula1>
-          <xm:sqref>I1:I296 I300:I329 I331:I340 I342:I1048576</xm:sqref>
+          <xm:sqref>I1:I296 I300:I329 I331:I340 I342:I357 I360:I366 I368 I370:I1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -31241,22 +32242,22 @@
         <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>631</v>
+        <v>662</v>
       </c>
       <c r="F1" t="s">
         <v>8</v>
       </c>
       <c r="G1" t="s">
-        <v>631</v>
+        <v>662</v>
       </c>
       <c r="I1" t="s">
-        <v>632</v>
+        <v>663</v>
       </c>
       <c r="K1" t="s">
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>633</v>
+        <v>664</v>
       </c>
       <c r="O1" t="s">
         <v>22</v>
@@ -31273,13 +32274,13 @@
         <v>572</v>
       </c>
       <c r="D2" t="s">
-        <v>634</v>
+        <v>665</v>
       </c>
       <c r="F2" t="s">
         <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>635</v>
+        <v>666</v>
       </c>
       <c r="I2" t="s">
         <v>516</v>
@@ -31305,13 +32306,13 @@
         <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>636</v>
+        <v>667</v>
       </c>
       <c r="F3" t="s">
         <v>185</v>
       </c>
       <c r="G3" t="s">
-        <v>637</v>
+        <v>668</v>
       </c>
       <c r="I3" t="s">
         <v>562</v>
@@ -31334,16 +32335,16 @@
         <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>638</v>
+        <v>669</v>
       </c>
       <c r="D4" t="s">
-        <v>639</v>
+        <v>670</v>
       </c>
       <c r="F4" t="s">
-        <v>640</v>
+        <v>671</v>
       </c>
       <c r="G4" t="s">
-        <v>641</v>
+        <v>672</v>
       </c>
       <c r="I4" t="s">
         <v>428</v>
@@ -31369,10 +32370,10 @@
         <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>642</v>
+        <v>673</v>
       </c>
       <c r="F5" t="s">
-        <v>643</v>
+        <v>674</v>
       </c>
       <c r="I5" t="s">
         <v>334</v>
@@ -31386,19 +32387,19 @@
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="2" t="s">
-        <v>644</v>
+        <v>675</v>
       </c>
       <c r="C6" t="s">
         <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>645</v>
+        <v>676</v>
       </c>
       <c r="F6" t="s">
         <v>103</v>
       </c>
       <c r="I6" t="s">
-        <v>646</v>
+        <v>677</v>
       </c>
       <c r="K6" t="s">
         <v>80</v>
@@ -31415,13 +32416,13 @@
         <v>366</v>
       </c>
       <c r="D7" t="s">
-        <v>647</v>
+        <v>678</v>
       </c>
       <c r="F7" t="s">
         <v>79</v>
       </c>
       <c r="I7" t="s">
-        <v>648</v>
+        <v>679</v>
       </c>
       <c r="K7" t="s">
         <v>105</v>
@@ -31435,7 +32436,7 @@
         <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>649</v>
+        <v>680</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
@@ -31444,7 +32445,7 @@
         <v>171</v>
       </c>
       <c r="K8" t="s">
-        <v>650</v>
+        <v>681</v>
       </c>
       <c r="M8" t="s">
         <v>436</v>
@@ -31455,10 +32456,10 @@
         <v>201</v>
       </c>
       <c r="C9" t="s">
-        <v>651</v>
+        <v>682</v>
       </c>
       <c r="D9" t="s">
-        <v>652</v>
+        <v>683</v>
       </c>
       <c r="F9" t="s">
         <v>61</v>
@@ -31481,13 +32482,13 @@
         <v>131</v>
       </c>
       <c r="D10" t="s">
-        <v>653</v>
+        <v>684</v>
       </c>
       <c r="F10" t="s">
         <v>470</v>
       </c>
       <c r="I10" t="s">
-        <v>654</v>
+        <v>685</v>
       </c>
       <c r="K10" t="s">
         <v>616</v>
@@ -31495,13 +32496,13 @@
     </row>
     <row r="11" spans="1:17">
       <c r="A11" t="s">
-        <v>655</v>
+        <v>686</v>
       </c>
       <c r="C11" t="s">
         <v>583</v>
       </c>
       <c r="D11" t="s">
-        <v>656</v>
+        <v>687</v>
       </c>
       <c r="K11" t="s">
         <v>61</v>
@@ -31512,15 +32513,15 @@
         <v>220</v>
       </c>
       <c r="C12" t="s">
-        <v>657</v>
+        <v>688</v>
       </c>
       <c r="D12" t="s">
-        <v>658</v>
+        <v>689</v>
       </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="1" t="s">
-        <v>659</v>
+        <v>690</v>
       </c>
       <c r="C13" t="s">
         <v>243</v>
@@ -31528,7 +32529,7 @@
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="2" t="s">
-        <v>660</v>
+        <v>691</v>
       </c>
       <c r="C14" t="s">
         <v>275</v>
@@ -31544,12 +32545,12 @@
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="2" t="s">
-        <v>661</v>
+        <v>692</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="1" t="s">
-        <v>662</v>
+        <v>693</v>
       </c>
     </row>
     <row r="18" spans="1:1">
@@ -31749,17 +32750,17 @@
     </row>
     <row r="5" spans="1:4">
       <c r="C5" t="s">
-        <v>663</v>
+        <v>694</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="B6" t="s">
-        <v>664</v>
+        <v>695</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>665</v>
+        <v>696</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -31778,17 +32779,17 @@
     </row>
     <row r="9" spans="1:4">
       <c r="C9" t="s">
-        <v>666</v>
+        <v>697</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="B10" t="s">
-        <v>667</v>
+        <v>698</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>668</v>
+        <v>699</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -31807,17 +32808,17 @@
     </row>
     <row r="13" spans="1:4">
       <c r="C13" t="s">
-        <v>669</v>
+        <v>700</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="B14" t="s">
-        <v>664</v>
+        <v>695</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>670</v>
+        <v>701</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -31836,17 +32837,17 @@
     </row>
     <row r="17" spans="1:4">
       <c r="C17" t="s">
-        <v>671</v>
+        <v>702</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="B18" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>673</v>
+        <v>704</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -31865,17 +32866,17 @@
     </row>
     <row r="21" spans="1:4">
       <c r="C21" t="s">
-        <v>674</v>
+        <v>705</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="B22" t="s">
-        <v>667</v>
+        <v>698</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>675</v>
+        <v>706</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -31894,17 +32895,17 @@
     </row>
     <row r="25" spans="1:4">
       <c r="C25" t="s">
-        <v>676</v>
+        <v>707</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="B26" t="s">
-        <v>664</v>
+        <v>695</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>677</v>
+        <v>708</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -31923,17 +32924,17 @@
     </row>
     <row r="29" spans="1:4">
       <c r="C29" t="s">
-        <v>678</v>
+        <v>709</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="B30" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>679</v>
+        <v>710</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -31952,17 +32953,17 @@
     </row>
     <row r="33" spans="1:4">
       <c r="C33" t="s">
-        <v>663</v>
+        <v>694</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="B34" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>680</v>
+        <v>711</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -31981,17 +32982,17 @@
     </row>
     <row r="37" spans="1:4">
       <c r="C37" t="s">
-        <v>681</v>
+        <v>712</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="B38" t="s">
-        <v>682</v>
+        <v>713</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>683</v>
+        <v>714</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -32010,17 +33011,17 @@
     </row>
     <row r="41" spans="1:4">
       <c r="C41" t="s">
-        <v>684</v>
+        <v>715</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="B42" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>685</v>
+        <v>716</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -32039,17 +33040,17 @@
     </row>
     <row r="45" spans="1:4">
       <c r="C45" t="s">
-        <v>686</v>
+        <v>717</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="B46" t="s">
-        <v>667</v>
+        <v>698</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>687</v>
+        <v>718</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -32068,17 +33069,17 @@
     </row>
     <row r="49" spans="1:4">
       <c r="C49" t="s">
-        <v>681</v>
+        <v>712</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="B50" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>688</v>
+        <v>719</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -32097,17 +33098,17 @@
     </row>
     <row r="53" spans="1:4">
       <c r="C53" t="s">
-        <v>689</v>
+        <v>720</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="B54" t="s">
-        <v>664</v>
+        <v>695</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>690</v>
+        <v>721</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -32126,17 +33127,17 @@
     </row>
     <row r="57" spans="1:4">
       <c r="C57" t="s">
-        <v>689</v>
+        <v>720</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="B58" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>691</v>
+        <v>722</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -32155,17 +33156,17 @@
     </row>
     <row r="61" spans="1:4">
       <c r="C61" t="s">
-        <v>671</v>
+        <v>702</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="B62" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" t="s">
-        <v>692</v>
+        <v>723</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -32184,17 +33185,17 @@
     </row>
     <row r="65" spans="1:4">
       <c r="C65" t="s">
-        <v>684</v>
+        <v>715</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="B66" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" t="s">
-        <v>693</v>
+        <v>724</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -32213,17 +33214,17 @@
     </row>
     <row r="69" spans="1:4">
       <c r="C69" t="s">
-        <v>689</v>
+        <v>720</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="B70" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" t="s">
-        <v>694</v>
+        <v>725</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -32242,22 +33243,22 @@
     </row>
     <row r="73" spans="1:4">
       <c r="C73" t="s">
-        <v>695</v>
+        <v>726</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="B74" t="s">
-        <v>672</v>
+        <v>703</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" t="s">
-        <v>696</v>
+        <v>727</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" t="s">
-        <v>697</v>
+        <v>728</v>
       </c>
     </row>
   </sheetData>

</xml_diff>